<commit_message>
added Veo Poster to screen 27, host pi5pm32
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/Poster/rt2026/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF0DEFA-28AE-AD4A-8DE8-C04806B1D715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="220" yWindow="600" windowWidth="30720" windowHeight="15280" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -19,12 +25,12 @@
     <sheet name="28937" sheetId="10" r:id="rId10"/>
     <sheet name="28938" sheetId="11" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="484">
   <si>
     <t>Key</t>
   </si>
@@ -1392,16 +1398,106 @@
   </si>
   <si>
     <t>Research Center for Nuclear Physics</t>
+  </si>
+  <si>
+    <t>pi5pm1</t>
+  </si>
+  <si>
+    <t>pi5pm2</t>
+  </si>
+  <si>
+    <t>pi5pm3</t>
+  </si>
+  <si>
+    <t>pi5pm4</t>
+  </si>
+  <si>
+    <t>pi5pm5</t>
+  </si>
+  <si>
+    <t>pi5pm6</t>
+  </si>
+  <si>
+    <t>pi5pm7</t>
+  </si>
+  <si>
+    <t>pi5pm8</t>
+  </si>
+  <si>
+    <t>pi5pm9</t>
+  </si>
+  <si>
+    <t>pi5pm10</t>
+  </si>
+  <si>
+    <t>pi5pm11</t>
+  </si>
+  <si>
+    <t>pi5pm12</t>
+  </si>
+  <si>
+    <t>pi5pm13</t>
+  </si>
+  <si>
+    <t>pi5pm14</t>
+  </si>
+  <si>
+    <t>pi5pm15</t>
+  </si>
+  <si>
+    <t>pi5pm16</t>
+  </si>
+  <si>
+    <t>pi5pm17</t>
+  </si>
+  <si>
+    <t>pi5pm18</t>
+  </si>
+  <si>
+    <t>pi5pm19</t>
+  </si>
+  <si>
+    <t>pi5pm20</t>
+  </si>
+  <si>
+    <t>pi5pm21</t>
+  </si>
+  <si>
+    <t>pi5pm22</t>
+  </si>
+  <si>
+    <t>pi5pm23</t>
+  </si>
+  <si>
+    <t>pi5pm24</t>
+  </si>
+  <si>
+    <t>pi5pm25</t>
+  </si>
+  <si>
+    <t>pi5pm26</t>
+  </si>
+  <si>
+    <t>pi5pm32</t>
+  </si>
+  <si>
+    <t>pi5pm33</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1427,21 +1523,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1479,7 +1584,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1513,6 +1618,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1547,9 +1653,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1722,15 +1829,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="100.7109375" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1738,7 +1845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1746,7 +1853,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1754,7 +1861,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1762,7 +1869,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1776,17 +1883,17 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -1806,7 +1913,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>62</v>
       </c>
@@ -1823,7 +1930,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>152</v>
       </c>
@@ -1840,7 +1947,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>162</v>
       </c>
@@ -1857,7 +1964,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>166</v>
       </c>
@@ -1874,7 +1981,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>178</v>
       </c>
@@ -1891,7 +1998,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>179</v>
       </c>
@@ -1908,7 +2015,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>180</v>
       </c>
@@ -1925,7 +2032,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>181</v>
       </c>
@@ -1942,7 +2049,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>182</v>
       </c>
@@ -1959,7 +2066,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>185</v>
       </c>
@@ -1976,7 +2083,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>190</v>
       </c>
@@ -1993,7 +2100,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>194</v>
       </c>
@@ -2010,7 +2117,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>200</v>
       </c>
@@ -2033,17 +2140,17 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -2063,7 +2170,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>73</v>
       </c>
@@ -2080,7 +2187,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>115</v>
       </c>
@@ -2097,7 +2204,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>134</v>
       </c>
@@ -2114,7 +2221,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>135</v>
       </c>
@@ -2131,7 +2238,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>136</v>
       </c>
@@ -2148,7 +2255,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>139</v>
       </c>
@@ -2165,7 +2272,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>147</v>
       </c>
@@ -2182,7 +2289,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>148</v>
       </c>
@@ -2199,7 +2306,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>149</v>
       </c>
@@ -2216,10 +2323,13 @@
         <v>447</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>150</v>
       </c>
+      <c r="B11">
+        <v>27</v>
+      </c>
       <c r="C11" t="s">
         <v>401</v>
       </c>
@@ -2233,7 +2343,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>153</v>
       </c>
@@ -2250,7 +2360,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>173</v>
       </c>
@@ -2267,7 +2377,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>189</v>
       </c>
@@ -2284,7 +2394,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>192</v>
       </c>
@@ -2301,7 +2411,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>197</v>
       </c>
@@ -2318,7 +2428,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>199</v>
       </c>
@@ -2335,7 +2445,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>207</v>
       </c>
@@ -2352,7 +2462,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>213</v>
       </c>
@@ -2369,7 +2479,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>216</v>
       </c>
@@ -2392,16 +2502,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" width="100.7109375" customWidth="1"/>
-    <col min="3" max="4" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.6640625" customWidth="1"/>
+    <col min="3" max="4" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -2415,7 +2525,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>28931</v>
       </c>
@@ -2429,7 +2539,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>28932</v>
       </c>
@@ -2443,7 +2553,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>28933</v>
       </c>
@@ -2457,7 +2567,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>28934</v>
       </c>
@@ -2471,7 +2581,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>28935</v>
       </c>
@@ -2485,7 +2595,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>28936</v>
       </c>
@@ -2499,7 +2609,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>28937</v>
       </c>
@@ -2513,18 +2623,18 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>28938</v>
       </c>
       <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" t="s">
-        <v>26</v>
+      <c r="C9" s="1">
+        <v>46140.475694444445</v>
+      </c>
+      <c r="D9" s="1">
+        <v>46162.520833333336</v>
       </c>
     </row>
   </sheetData>
@@ -2533,14 +2643,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="20.7109375" customWidth="1"/>
+    <col min="1" max="2" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -2548,23 +2658,248 @@
         <v>28</v>
       </c>
     </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>456</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>457</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>458</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>460</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>461</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>462</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>463</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>464</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>465</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>466</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>467</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>468</v>
+      </c>
+      <c r="B14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>469</v>
+      </c>
+      <c r="B15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>470</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>471</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>472</v>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>473</v>
+      </c>
+      <c r="B19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>474</v>
+      </c>
+      <c r="B20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>475</v>
+      </c>
+      <c r="B21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>476</v>
+      </c>
+      <c r="B22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>477</v>
+      </c>
+      <c r="B23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>478</v>
+      </c>
+      <c r="B24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>479</v>
+      </c>
+      <c r="B25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>480</v>
+      </c>
+      <c r="B26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>481</v>
+      </c>
+      <c r="B27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>482</v>
+      </c>
+      <c r="B28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>483</v>
+      </c>
+      <c r="B29">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -2584,7 +2919,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>12</v>
       </c>
@@ -2601,7 +2936,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>16</v>
       </c>
@@ -2615,7 +2950,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>26</v>
       </c>
@@ -2632,7 +2967,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>28</v>
       </c>
@@ -2649,7 +2984,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>188</v>
       </c>
@@ -2663,7 +2998,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>204</v>
       </c>
@@ -2686,17 +3021,17 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -2716,7 +3051,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>6</v>
       </c>
@@ -2733,7 +3068,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>19</v>
       </c>
@@ -2750,7 +3085,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>22</v>
       </c>
@@ -2767,7 +3102,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>32</v>
       </c>
@@ -2784,7 +3119,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>34</v>
       </c>
@@ -2801,7 +3136,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>38</v>
       </c>
@@ -2818,7 +3153,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>39</v>
       </c>
@@ -2835,7 +3170,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>40</v>
       </c>
@@ -2852,7 +3187,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>43</v>
       </c>
@@ -2869,7 +3204,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>55</v>
       </c>
@@ -2886,7 +3221,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>59</v>
       </c>
@@ -2903,7 +3238,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>87</v>
       </c>
@@ -2920,7 +3255,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>94</v>
       </c>
@@ -2937,7 +3272,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>101</v>
       </c>
@@ -2954,7 +3289,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>105</v>
       </c>
@@ -2968,7 +3303,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>108</v>
       </c>
@@ -2985,7 +3320,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>129</v>
       </c>
@@ -2999,7 +3334,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>130</v>
       </c>
@@ -3013,7 +3348,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>132</v>
       </c>
@@ -3030,7 +3365,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>137</v>
       </c>
@@ -3047,7 +3382,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>140</v>
       </c>
@@ -3064,7 +3399,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>142</v>
       </c>
@@ -3081,7 +3416,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>160</v>
       </c>
@@ -3098,7 +3433,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>168</v>
       </c>
@@ -3115,7 +3450,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>174</v>
       </c>
@@ -3132,7 +3467,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>177</v>
       </c>
@@ -3155,17 +3490,17 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -3185,7 +3520,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>27</v>
       </c>
@@ -3202,7 +3537,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>52</v>
       </c>
@@ -3219,7 +3554,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>61</v>
       </c>
@@ -3236,7 +3571,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>75</v>
       </c>
@@ -3253,7 +3588,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>99</v>
       </c>
@@ -3270,7 +3605,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>102</v>
       </c>
@@ -3287,7 +3622,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>119</v>
       </c>
@@ -3304,7 +3639,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>124</v>
       </c>
@@ -3321,7 +3656,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>127</v>
       </c>
@@ -3335,7 +3670,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>131</v>
       </c>
@@ -3349,7 +3684,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>145</v>
       </c>
@@ -3366,7 +3701,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>161</v>
       </c>
@@ -3383,7 +3718,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>165</v>
       </c>
@@ -3397,7 +3732,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>196</v>
       </c>
@@ -3411,7 +3746,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>218</v>
       </c>
@@ -3425,7 +3760,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>219</v>
       </c>
@@ -3445,17 +3780,17 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -3475,7 +3810,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>96</v>
       </c>
@@ -3492,7 +3827,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>100</v>
       </c>
@@ -3509,7 +3844,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>114</v>
       </c>
@@ -3526,7 +3861,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>141</v>
       </c>
@@ -3540,7 +3875,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>144</v>
       </c>
@@ -3557,7 +3892,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>146</v>
       </c>
@@ -3574,7 +3909,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>151</v>
       </c>
@@ -3591,7 +3926,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>155</v>
       </c>
@@ -3605,7 +3940,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>156</v>
       </c>
@@ -3622,7 +3957,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>158</v>
       </c>
@@ -3639,7 +3974,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>159</v>
       </c>
@@ -3656,7 +3991,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>167</v>
       </c>
@@ -3673,7 +4008,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>175</v>
       </c>
@@ -3690,7 +4025,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>184</v>
       </c>
@@ -3707,7 +4042,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>210</v>
       </c>
@@ -3721,7 +4056,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>214</v>
       </c>
@@ -3738,7 +4073,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>215</v>
       </c>
@@ -3761,17 +4096,17 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -3791,7 +4126,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>17</v>
       </c>
@@ -3808,7 +4143,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>20</v>
       </c>
@@ -3825,7 +4160,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>21</v>
       </c>
@@ -3842,7 +4177,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>35</v>
       </c>
@@ -3856,7 +4191,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>42</v>
       </c>
@@ -3873,7 +4208,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>46</v>
       </c>
@@ -3887,7 +4222,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>49</v>
       </c>
@@ -3901,7 +4236,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>51</v>
       </c>
@@ -3915,7 +4250,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>81</v>
       </c>
@@ -3932,7 +4267,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>82</v>
       </c>
@@ -3949,7 +4284,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>84</v>
       </c>
@@ -3963,7 +4298,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>86</v>
       </c>
@@ -3980,7 +4315,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>103</v>
       </c>
@@ -3997,7 +4332,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>106</v>
       </c>
@@ -4014,7 +4349,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>116</v>
       </c>
@@ -4031,7 +4366,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>126</v>
       </c>
@@ -4054,17 +4389,17 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -4084,7 +4419,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>23</v>
       </c>
@@ -4101,7 +4436,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>29</v>
       </c>
@@ -4118,7 +4453,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>31</v>
       </c>
@@ -4135,7 +4470,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>37</v>
       </c>
@@ -4152,7 +4487,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>64</v>
       </c>
@@ -4169,7 +4504,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>65</v>
       </c>
@@ -4183,7 +4518,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>68</v>
       </c>
@@ -4200,7 +4535,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>69</v>
       </c>
@@ -4214,7 +4549,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>76</v>
       </c>
@@ -4231,7 +4566,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>85</v>
       </c>
@@ -4248,7 +4583,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>89</v>
       </c>
@@ -4265,7 +4600,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>95</v>
       </c>
@@ -4282,7 +4617,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>104</v>
       </c>
@@ -4299,7 +4634,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>112</v>
       </c>
@@ -4316,7 +4651,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>123</v>
       </c>
@@ -4330,7 +4665,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
fixed problem with daytime
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/Poster/rt2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF0DEFA-28AE-AD4A-8DE8-C04806B1D715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2323F32-AF11-5A41-9BA5-615480F1E153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="600" windowWidth="30720" windowHeight="15280" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="220" yWindow="600" windowWidth="30720" windowHeight="15280" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="484">
   <si>
     <t>Key</t>
   </si>
@@ -1523,9 +1523,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2328,7 +2327,7 @@
         <v>150</v>
       </c>
       <c r="B11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
         <v>401</v>
@@ -2630,11 +2629,11 @@
       <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="1">
-        <v>46140.475694444445</v>
-      </c>
-      <c r="D9" s="1">
-        <v>46162.520833333336</v>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
three poster, missing qrcodes, updated roster
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marco/work/git/rt2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ABF08D4-BD60-8D4A-9D77-77DF4C052C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{747DC37F-FA9B-DF42-91F6-1FDB1DABFD27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="24360" windowHeight="17160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="14680" windowHeight="17160" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="479">
   <si>
     <t>Key</t>
   </si>
@@ -68,6 +68,54 @@
     <t>Session end</t>
   </si>
   <si>
+    <t>Emerging Technologies, New Standards, Feedback on Experience &amp; Industry - PS</t>
+  </si>
+  <si>
+    <t>Front-End Electronics, Fast Digitizers, Fast Transfer Links &amp; Networks - PS: A</t>
+  </si>
+  <si>
+    <t>AI, Machine Learning, Real Time Simulation, Intelligent Signal Processing - PS</t>
+  </si>
+  <si>
+    <t>Real Time Diagnostics, Digital Twin, Control, Monitoring, Safety and Security - PS: B</t>
+  </si>
+  <si>
+    <t>Data Acquisition and Trigger Architectures - PS: A</t>
+  </si>
+  <si>
+    <t>Real Time Diagnostics, Digital Twin, Control, Monitoring, Safety and Security - PS: A</t>
+  </si>
+  <si>
+    <t>Front-End Electronics, Fast Digitizers, Fast Transfer Links &amp; Networks - PS: B</t>
+  </si>
+  <si>
+    <t>Data Acquisition and Trigger Architectures - PS: B</t>
+  </si>
+  <si>
+    <t>2026-05-25 14:45:00</t>
+  </si>
+  <si>
+    <t>2026-05-27 11:05:00</t>
+  </si>
+  <si>
+    <t>2026-05-26 11:25:00</t>
+  </si>
+  <si>
+    <t>2026-05-28 11:25:00</t>
+  </si>
+  <si>
+    <t>2026-05-25 15:45:00</t>
+  </si>
+  <si>
+    <t>2026-05-27 12:05:00</t>
+  </si>
+  <si>
+    <t>2026-05-26 12:30:00</t>
+  </si>
+  <si>
+    <t>2026-05-28 12:30:00</t>
+  </si>
+  <si>
     <t>Hostname</t>
   </si>
   <si>
@@ -146,12 +194,18 @@
     <t>European Spallation Source</t>
   </si>
   <si>
+    <t>KIT</t>
+  </si>
+  <si>
     <t>Science and Technology Facilities Council STFC (GB)</t>
   </si>
   <si>
     <t>Max-Planck-Institute for Plasma Physics</t>
   </si>
   <si>
+    <t>Energy Sciences Network</t>
+  </si>
+  <si>
     <t>SkuTek Instrumentation</t>
   </si>
   <si>
@@ -278,7 +332,7 @@
     <t>jiayun</t>
   </si>
   <si>
-    <t>chunlai</t>
+    <t>Chunlai</t>
   </si>
   <si>
     <t>Giovanni</t>
@@ -419,6 +473,9 @@
     <t>山东大学</t>
   </si>
   <si>
+    <t>Central China Normal University</t>
+  </si>
+  <si>
     <t>CAEN S.p.A.</t>
   </si>
   <si>
@@ -431,9 +488,6 @@
     <t>RIKEN Nishina Center</t>
   </si>
   <si>
-    <t>Central China Normal University</t>
-  </si>
-  <si>
     <t>Institute of High Energy Physics</t>
   </si>
   <si>
@@ -581,12 +635,21 @@
     <t>Facility for Rare Isotope Beams @ Michigan State University</t>
   </si>
   <si>
+    <t>Lawrence Berkley National Laboratory</t>
+  </si>
+  <si>
+    <t>Technische Hochschule Ostwestfalen</t>
+  </si>
+  <si>
     <t>INFN Pisa</t>
   </si>
   <si>
     <t>Universite Libre de Bruxelles (BE)</t>
   </si>
   <si>
+    <t>Universitat de València</t>
+  </si>
+  <si>
     <t>A Low-Latency Distributed Machine-Protection System for the PIP-II Linear Accelerator</t>
   </si>
   <si>
@@ -644,10 +707,10 @@
     <t>Emmanuel</t>
   </si>
   <si>
-    <t>TIANYI</t>
-  </si>
-  <si>
-    <t>Xiaochuan</t>
+    <t>Tianyi</t>
+  </si>
+  <si>
+    <t>Huang</t>
   </si>
   <si>
     <t>Wanook</t>
@@ -656,15 +719,12 @@
     <t>Arjana</t>
   </si>
   <si>
-    <t>xiaofeng</t>
+    <t>Xiaofeng</t>
   </si>
   <si>
     <t>Tianjue</t>
   </si>
   <si>
-    <t>Tianyi</t>
-  </si>
-  <si>
     <t>Si</t>
   </si>
   <si>
@@ -689,451 +749,436 @@
     <t>Uwitonze</t>
   </si>
   <si>
-    <t>JIANG</t>
+    <t>Jiang</t>
+  </si>
+  <si>
+    <t>Ji</t>
+  </si>
+  <si>
+    <t>Kolnikaj</t>
+  </si>
+  <si>
+    <t>Zhu</t>
+  </si>
+  <si>
+    <t>Ma</t>
+  </si>
+  <si>
+    <t>Gao</t>
+  </si>
+  <si>
+    <t>Kleines</t>
+  </si>
+  <si>
+    <t>Ferron</t>
+  </si>
+  <si>
+    <t>Weldon</t>
+  </si>
+  <si>
+    <t>Fermi National Accelerator Lab. (US)</t>
+  </si>
+  <si>
+    <t>National Institute for Nuclear Physics, Section of Pisa, Pisa, Italy</t>
+  </si>
+  <si>
+    <t>China Institute of Atomic Energy</t>
+  </si>
+  <si>
+    <t>IHEP - Chinese Academy of Sciences</t>
+  </si>
+  <si>
+    <t>Korea Atomic Energy Research Institute</t>
+  </si>
+  <si>
+    <t>University of Glasgow</t>
+  </si>
+  <si>
+    <t>Tianjin University of Technology</t>
+  </si>
+  <si>
+    <t>Forschungszentrum Jülich</t>
+  </si>
+  <si>
+    <t>Consorzio RFX</t>
+  </si>
+  <si>
+    <t>CEA, Cadarache</t>
+  </si>
+  <si>
+    <t>Real Time Data Acquisition for Atmospheric muography based on the Thin Gap Chamber</t>
+  </si>
+  <si>
+    <t>MicroTCA-based low latency data streaming and processing architecture using UDP offload and Time Sensitive Networking</t>
+  </si>
+  <si>
+    <t>Development of the IDROGEN White Rabbit system for SuperKEKB and future projects at KEK</t>
+  </si>
+  <si>
+    <t>Streaming Readout DAQ Systems for High-Luminosity Electron-Beam Experiments</t>
+  </si>
+  <si>
+    <t>CODA SRO DAQ with Real-Time Data Processing Components</t>
+  </si>
+  <si>
+    <t>A versatile, high accuracy, pulsed measurement device</t>
+  </si>
+  <si>
+    <t>Exploration on Quasi-Steady-State Real-Time Data Access for EAST Tokamak</t>
+  </si>
+  <si>
+    <t>FPGA-Accelerated Pattern Recognition for the ATLAS Event Filter at the HL-LHC</t>
+  </si>
+  <si>
+    <t>Regional reconstruction of tracks for the ATLAS Event Filter using GPU accelerators</t>
+  </si>
+  <si>
+    <t>A Heterogeneous Software Framework Design for the Full Software Trigger at CEPC</t>
+  </si>
+  <si>
+    <t>Development of a Coincidence Measurement System for Scattered and Decay Particles Using a Streaming DAQ and Digitizers</t>
+  </si>
+  <si>
+    <t>Timing and Slow Control backend for CMS Drift Tube On Board electronics</t>
+  </si>
+  <si>
+    <t>Design and Results of a Radiation Test System for SEE and TID Assessment of the VLAST-P CsI(Tl) Calorimeter Readout Electronics</t>
+  </si>
+  <si>
+    <t>Jia</t>
+  </si>
+  <si>
+    <t>Hiroshi</t>
+  </si>
+  <si>
+    <t>Fabio</t>
+  </si>
+  <si>
+    <t>Mario</t>
+  </si>
+  <si>
+    <t>Ying</t>
+  </si>
+  <si>
+    <t>Priya</t>
+  </si>
+  <si>
+    <t>Benjamin Michael</t>
+  </si>
+  <si>
+    <t>Shotaro</t>
+  </si>
+  <si>
+    <t>Antonio</t>
+  </si>
+  <si>
+    <t>JiaAo</t>
+  </si>
+  <si>
+    <t>Piñas-Hugueruela</t>
+  </si>
+  <si>
+    <t>Kaji</t>
+  </si>
+  <si>
+    <t>Rossi</t>
+  </si>
+  <si>
+    <t>Abbott</t>
+  </si>
+  <si>
+    <t>Jurcevic</t>
+  </si>
+  <si>
+    <t>Sundararajan</t>
+  </si>
+  <si>
+    <t>Wynne</t>
+  </si>
+  <si>
+    <t>Maesato</t>
+  </si>
+  <si>
+    <t>Bergnoli</t>
+  </si>
+  <si>
+    <t>Universidad Politecnica de Madrid</t>
+  </si>
+  <si>
+    <t>INFN</t>
+  </si>
+  <si>
+    <t>JLAB</t>
+  </si>
+  <si>
+    <t>Paul Scherrer Institut</t>
+  </si>
+  <si>
+    <t>Hefei Institutes of Physical Science</t>
+  </si>
+  <si>
+    <t>University of California Irvine (US)</t>
+  </si>
+  <si>
+    <t>The University of Edinburgh (GB)</t>
+  </si>
+  <si>
+    <t>The Institute of High Energy Physics of the Chinese Academy of Sciences</t>
+  </si>
+  <si>
+    <t>The University of Osaka</t>
+  </si>
+  <si>
+    <t>Universita e INFN, Padova (IT)</t>
+  </si>
+  <si>
+    <t>Shape-factor analysis of real-time, in-situ photon-depth spectra for land quality β--emitter assay</t>
+  </si>
+  <si>
+    <t>The ATLAS Forward Proton (AFP) sub-detector and the adverse effects of radiation from Large Hadron Collider (LHC) collimators during pp-collisions at 13.6 TeV</t>
+  </si>
+  <si>
+    <t>Design and Implementation of a Distributed  Detector Control System for the JUNO Experiment</t>
+  </si>
+  <si>
+    <t>Electronics for Two-Dimensional Magnetic-Field Measurement in a Polarized-Light Helium Optically Pumped Magnetometer</t>
+  </si>
+  <si>
+    <t>FPGA-based  online monitoring  for  triggerless readout system in dark matter experiment</t>
+  </si>
+  <si>
+    <t>Data flow management and service of Lingshu plasma control system</t>
+  </si>
+  <si>
+    <t>Low-latency digital control of an all-in-fiber phase noise reduction loop for VIRGO Squeezer</t>
+  </si>
+  <si>
+    <t>Enhancements of the central Safety System for Wendelstein 7-X operational phase OP2.4</t>
+  </si>
+  <si>
+    <t>Development of algorithms for the end-end system simulation, mode analysis and performance optimization for a generic and multi-tokamak high-frequency magnetic diagnostic system</t>
+  </si>
+  <si>
+    <t>A Low-Dead Time FPGA-TDC for Optical Beam-Loss Monitor System</t>
+  </si>
+  <si>
+    <t>High‑Voltage System control for the ICARUS experiment at Fermilab</t>
+  </si>
+  <si>
+    <t>Deep Fusion Attention Transfer Learning Method for Rotating Machinery Fault Diagnosis Based on Two Stage Neural Network</t>
+  </si>
+  <si>
+    <t>UPGRADED CONTROL SYSTEM FOR THE ELECTRON CYCLOTRON HEATING EXPANSION SYSTEM ON EAST</t>
+  </si>
+  <si>
+    <t>Development of a Portable Real-Time Radiation Measurement Technology for Digital Twin Based Plant Situation Monitoring</t>
+  </si>
+  <si>
+    <t>Data Orchestration and Large Model-Driven Interactive Diagnosis for LHAASO Operational Data</t>
+  </si>
+  <si>
+    <t>Distributed Modeling and Simulation Methods for Tokamak Simulation Systems</t>
+  </si>
+  <si>
+    <t>Kate</t>
+  </si>
+  <si>
+    <t>Marko</t>
+  </si>
+  <si>
+    <t>Mei</t>
+  </si>
+  <si>
+    <t>Xuan</t>
+  </si>
+  <si>
+    <t>Jianqiu</t>
+  </si>
+  <si>
+    <t>Marco</t>
+  </si>
+  <si>
+    <t>Jörg</t>
+  </si>
+  <si>
+    <t>Duccio</t>
+  </si>
+  <si>
+    <t>Yuchen</t>
+  </si>
+  <si>
+    <t>Shaoqing</t>
+  </si>
+  <si>
+    <t>Weiye</t>
+  </si>
+  <si>
+    <t>Hyeoung Woo</t>
+  </si>
+  <si>
+    <t>Heru</t>
+  </si>
+  <si>
+    <t>Williams</t>
+  </si>
+  <si>
+    <t>Milovanovic</t>
+  </si>
+  <si>
+    <t>Ye</t>
+  </si>
+  <si>
+    <t>Mastroianni</t>
+  </si>
+  <si>
+    <t>Toffano</t>
+  </si>
+  <si>
+    <t>Schacht</t>
+  </si>
+  <si>
+    <t>Testa</t>
+  </si>
+  <si>
+    <t>Gioiosa</t>
+  </si>
+  <si>
+    <t>Park</t>
+  </si>
+  <si>
+    <t>Guo</t>
+  </si>
+  <si>
+    <t>Lancaster University</t>
+  </si>
+  <si>
+    <t>Justus-Liebig-Universitaet Giessen (DE)</t>
+  </si>
+  <si>
+    <t>IHEP</t>
+  </si>
+  <si>
+    <t>INFN Napoli</t>
+  </si>
+  <si>
+    <t>Institute of Plasma Physics, Chinese Academy of Sciences</t>
+  </si>
+  <si>
+    <t>Max-Planck-Institut für Plasmaphysik</t>
+  </si>
+  <si>
+    <t>EPFL</t>
+  </si>
+  <si>
+    <t>Anhui University</t>
+  </si>
+  <si>
+    <t>University of Molise &amp; INFN Roma Tor Vergata</t>
+  </si>
+  <si>
+    <t>Institute of Energy Hefei Comprehensive National Science Center</t>
+  </si>
+  <si>
+    <t>Central Research Institute, Korea Hydro &amp; Nuclear Power Co., Ltd.</t>
+  </si>
+  <si>
+    <t>Institute of Energy, Hefei Comprehensive National Science Center</t>
+  </si>
+  <si>
+    <t>A Modular MPSoC Platform for Real-time Data Processing for Climate Observation Instruments</t>
+  </si>
+  <si>
+    <t>Operations and Performance of the ATLAS Tile Calorimeter Phase-II Upgrade Demonstrator in Run 3</t>
+  </si>
+  <si>
+    <t>A Timing Measurement Prototype for LGAD Using the LATRIC ASIC</t>
+  </si>
+  <si>
+    <t>Toward Efficient Wireless Monitoring in Nuclear Facilities Based on Named Data Networking</t>
+  </si>
+  <si>
+    <t>A Multi-Mode Waveform Digitization System Based on Switched Capacitor Array Chips</t>
+  </si>
+  <si>
+    <t>Design of Prototype Readout Electronics of the High Counting Rate Main Drift Chamber in Particle Physics Experiments</t>
+  </si>
+  <si>
+    <t>Prototype Readout Electronics System for a LET Spectrometer in Space Radiation</t>
+  </si>
+  <si>
+    <t>A Full on-Chip LDO Regulator with self-adapting compensation networks for Front-end Readout Circuit</t>
+  </si>
+  <si>
+    <t>The μMUX readout electronic system of the AliCPT</t>
+  </si>
+  <si>
+    <t>Low-Noise Room-Temperature Readout Electronics for TDM-SQUID TES Arrays in the AliCPT-40G Telescope</t>
+  </si>
+  <si>
+    <t>A 14-bit 100 Ms/s Pipeline ADC for Silicon Pixel Sensor in Gaseous Detectors</t>
+  </si>
+  <si>
+    <t>Performance Test of the SAMIDARE Board with Mini-TPC using heavy-Ion Beams</t>
+  </si>
+  <si>
+    <t>Design of a Novel Pipelined SAR ADC for Multi-channel Front-end ASICs</t>
+  </si>
+  <si>
+    <t>Georg</t>
+  </si>
+  <si>
+    <t>Fernando</t>
+  </si>
+  <si>
+    <t>Ziwen</t>
+  </si>
+  <si>
+    <t>Dingjun</t>
+  </si>
+  <si>
+    <t>Yilin</t>
+  </si>
+  <si>
+    <t>Wenrui</t>
+  </si>
+  <si>
+    <t>Xiayu</t>
+  </si>
+  <si>
+    <t>Xiangxiang</t>
+  </si>
+  <si>
+    <t>Tangchong</t>
+  </si>
+  <si>
+    <t>Haoqing</t>
+  </si>
+  <si>
+    <t>Fumitaka</t>
+  </si>
+  <si>
+    <t>Schardt</t>
+  </si>
+  <si>
+    <t>Carrio Argos</t>
+  </si>
+  <si>
+    <t>Lu</t>
+  </si>
+  <si>
+    <t>Sun</t>
+  </si>
+  <si>
+    <t>Ren</t>
+  </si>
+  <si>
+    <t>Kuang</t>
   </si>
   <si>
     <t>Xie</t>
   </si>
   <si>
-    <t>Ji</t>
-  </si>
-  <si>
-    <t>Kolnikaj</t>
-  </si>
-  <si>
-    <t>zhu</t>
-  </si>
-  <si>
-    <t>Jiang</t>
-  </si>
-  <si>
-    <t>MA</t>
-  </si>
-  <si>
-    <t>Gao</t>
-  </si>
-  <si>
-    <t>Kleines</t>
-  </si>
-  <si>
-    <t>Ferron</t>
-  </si>
-  <si>
-    <t>Weldon</t>
-  </si>
-  <si>
-    <t>Fermi National Accelerator Lab. (US)</t>
-  </si>
-  <si>
-    <t>National Institute for Nuclear Physics, Section of Pisa, Pisa, Italy</t>
-  </si>
-  <si>
-    <t>IHEP</t>
-  </si>
-  <si>
-    <t>Korea Atomic Energy Research Institute</t>
-  </si>
-  <si>
-    <t>University of Glasgow</t>
-  </si>
-  <si>
-    <t>China Institute of Atomic Energy</t>
-  </si>
-  <si>
-    <t>Tianjin University of Technology</t>
-  </si>
-  <si>
-    <t>Consorzio RFX</t>
-  </si>
-  <si>
-    <t>CEA, Cadarache</t>
-  </si>
-  <si>
-    <t>Design of the Global Timing Unit (GTU) for ePIC</t>
-  </si>
-  <si>
-    <t>Real Time Data Acquisition for Atmospheric muography based on the Thin Gap Chamber</t>
-  </si>
-  <si>
-    <t>MicroTCA-based low latency data streaming and processing architecture using UDP offload and Time Sensitive Networking</t>
-  </si>
-  <si>
-    <t>Development of the IDROGEN White Rabbit system for SuperKEKB and future projects at KEK</t>
-  </si>
-  <si>
-    <t>Streaming Readout DAQ Systems for High-Luminosity Electron-Beam Experiments</t>
-  </si>
-  <si>
-    <t>CODA SRO DAQ with Real-Time Data Processing Components</t>
-  </si>
-  <si>
-    <t>A versatile, high accuracy, pulsed measurement device</t>
-  </si>
-  <si>
-    <t>Exploration on Quasi-Steady-State Real-Time Data Access for EAST Tokamak</t>
-  </si>
-  <si>
-    <t>FPGA-Accelerated Pattern Recognition for the ATLAS Event Filter at the HL-LHC</t>
-  </si>
-  <si>
-    <t>Regional reconstruction of tracks for the ATLAS Event Filter using GPU accelerators</t>
-  </si>
-  <si>
-    <t>A Heterogeneous Software Framework Design for the Full Software Trigger at CEPC</t>
-  </si>
-  <si>
-    <t>Development of a Coincidence Measurement System for Scattered and Decay Particles Using a Streaming DAQ and Digitizers</t>
-  </si>
-  <si>
-    <t>Timing and Slow Control backend for CMS Drift Tube On Board electronics</t>
-  </si>
-  <si>
-    <t>Design and Results of a Radiation Test System for SEE and TID Assessment of the VLAST-P CsI(Tl) Calorimeter Readout Electronics</t>
-  </si>
-  <si>
-    <t>William</t>
-  </si>
-  <si>
-    <t>Jia</t>
-  </si>
-  <si>
-    <t>ALEJANDRO</t>
-  </si>
-  <si>
-    <t>Hiroshi</t>
-  </si>
-  <si>
-    <t>Fabio</t>
-  </si>
-  <si>
-    <t>Mario</t>
-  </si>
-  <si>
-    <t>Ying</t>
-  </si>
-  <si>
-    <t>Priya</t>
-  </si>
-  <si>
-    <t>Benjamin Michael</t>
-  </si>
-  <si>
-    <t>xu</t>
-  </si>
-  <si>
-    <t>Shotaro</t>
-  </si>
-  <si>
-    <t>Antonio</t>
-  </si>
-  <si>
-    <t>JiaAo</t>
-  </si>
-  <si>
-    <t>Gu</t>
-  </si>
-  <si>
-    <t>PIÑAS-HIGUERUELA</t>
-  </si>
-  <si>
-    <t>Kaji</t>
-  </si>
-  <si>
-    <t>Rossi</t>
-  </si>
-  <si>
-    <t>Abbott</t>
-  </si>
-  <si>
-    <t>Jurcevic</t>
-  </si>
-  <si>
-    <t>Sundararajan</t>
-  </si>
-  <si>
-    <t>Wynne</t>
-  </si>
-  <si>
-    <t>zhang</t>
-  </si>
-  <si>
-    <t>Maesato</t>
-  </si>
-  <si>
-    <t>Bergnoli</t>
-  </si>
-  <si>
-    <t>Jefferson Lab</t>
-  </si>
-  <si>
-    <t>Universidad Politecnica de Madrid</t>
-  </si>
-  <si>
-    <t>INFN</t>
-  </si>
-  <si>
-    <t>University of California Irvine (US)</t>
-  </si>
-  <si>
-    <t>The University of Edinburgh (GB)</t>
-  </si>
-  <si>
-    <t>The Institute of High Energy Physics of the Chinese Academy of Sciences</t>
-  </si>
-  <si>
-    <t>The University of Osaka</t>
-  </si>
-  <si>
-    <t>Universita e INFN, Padova (IT)</t>
-  </si>
-  <si>
-    <t>Shape-factor analysis of real-time, in-situ photon-depth spectra for land quality β--emitter assay</t>
-  </si>
-  <si>
-    <t>The ATLAS Forward Proton (AFP) sub-detector and the adverse effects of radiation from Large Hadron Collider (LHC) collimators during pp-collisions at 13.6 TeV</t>
-  </si>
-  <si>
-    <t>Design and Implementation of a Distributed  Detector Control System for the JUNO Experiment</t>
-  </si>
-  <si>
-    <t>Electronics for Two-Dimensional Magnetic-Field Measurement in a Polarized-Light Helium Optically Pumped Magnetometer</t>
-  </si>
-  <si>
-    <t>FPGA-based  online monitoring  for  triggerless readout system in dark matter experiment</t>
-  </si>
-  <si>
-    <t>Data flow management and service of Lingshu plasma control system</t>
-  </si>
-  <si>
-    <t>Low-latency digital control of an all-in-fiber phase noise reduction loop for VIRGO Squeezer</t>
-  </si>
-  <si>
-    <t>Enhancements of the central Safety System for Wendelstein 7-X operational phase OP2.4</t>
-  </si>
-  <si>
-    <t>Development of algorithms for the end-end system simulation, mode analysis and performance optimization for a generic and multi-tokamak high-frequency magnetic diagnostic system</t>
-  </si>
-  <si>
-    <t>A Low-Dead Time FPGA-TDC for Optical Beam-Loss Monitor System</t>
-  </si>
-  <si>
-    <t>High‑Voltage System control for the ICARUS experiment at Fermilab</t>
-  </si>
-  <si>
-    <t>Deep Fusion Attention Transfer Learning Method for Rotating Machinery Fault Diagnosis Based on Two Stage Neural Network</t>
-  </si>
-  <si>
-    <t>UPGRADED CONTROL SYSTEM FOR THE ELECTRON CYCLOTRON HEATING EXPANSION SYSTEM ON EAST</t>
-  </si>
-  <si>
-    <t>Development of a Portable Real-Time Radiation Measurement Technology for Digital Twin Based Plant Situation Monitoring</t>
-  </si>
-  <si>
-    <t>Data Orchestration and Large Model-Driven Interactive Diagnosis for LHAASO Operational Data</t>
-  </si>
-  <si>
-    <t>Distributed Modeling and Simulation Methods for Tokamak Simulation Systems</t>
-  </si>
-  <si>
-    <t>Kate</t>
-  </si>
-  <si>
-    <t>Marko</t>
-  </si>
-  <si>
-    <t>Mei</t>
-  </si>
-  <si>
-    <t>Xuan</t>
-  </si>
-  <si>
-    <t>jq</t>
-  </si>
-  <si>
-    <t>Marco</t>
-  </si>
-  <si>
-    <t>Jörg</t>
-  </si>
-  <si>
-    <t>Duccio</t>
-  </si>
-  <si>
-    <t>Yuchen</t>
-  </si>
-  <si>
-    <t>Shaoqing</t>
-  </si>
-  <si>
-    <t>Weiye</t>
-  </si>
-  <si>
-    <t>HyeoungWoo</t>
-  </si>
-  <si>
-    <t>Huang</t>
-  </si>
-  <si>
-    <t>Heru</t>
-  </si>
-  <si>
-    <t>Williams</t>
-  </si>
-  <si>
-    <t>Milovanovic</t>
-  </si>
-  <si>
-    <t>YE</t>
-  </si>
-  <si>
-    <t>Mastroianni</t>
-  </si>
-  <si>
-    <t>Toffano</t>
-  </si>
-  <si>
-    <t>Schacht</t>
-  </si>
-  <si>
-    <t>Testa</t>
-  </si>
-  <si>
-    <t>Gioiosa</t>
-  </si>
-  <si>
-    <t>Park</t>
-  </si>
-  <si>
-    <t>Guo</t>
-  </si>
-  <si>
-    <t>Lancaster University</t>
-  </si>
-  <si>
-    <t>Justus-Liebig-Universitaet Giessen (DE)</t>
-  </si>
-  <si>
-    <t>INFN Napoli</t>
-  </si>
-  <si>
-    <t>EPFL</t>
-  </si>
-  <si>
-    <t>Anhui university</t>
-  </si>
-  <si>
-    <t>University of Molise &amp; INFN Roma Tor Vergata</t>
-  </si>
-  <si>
-    <t>Institute of Energy Hefei Comprehensive National Science Center</t>
-  </si>
-  <si>
-    <t>Institute of Plasma Physics, Chinese Academy of Sciences</t>
-  </si>
-  <si>
-    <t>Central Research Institute, Korea Hydro &amp; Nuclear Power Co., Ltd.</t>
-  </si>
-  <si>
-    <t>Institute of Energy, Hefei Comprehensive National Science Center</t>
-  </si>
-  <si>
-    <t>A Modular MPSoC Platform for Real-time Data Processing for Climate Observation Instruments</t>
-  </si>
-  <si>
-    <t>Operations and Performance of the ATLAS Tile Calorimeter Phase-II Upgrade Demonstrator in Run 3</t>
-  </si>
-  <si>
-    <t>A Timing Measurement Prototype for LGAD Using the LATRIC ASIC</t>
-  </si>
-  <si>
-    <t>Toward Efficient Wireless Monitoring in Nuclear Facilities Based on Named Data Networking</t>
-  </si>
-  <si>
-    <t>A Multi-Mode Waveform Digitization System Based on Switched Capacitor Array Chips</t>
-  </si>
-  <si>
-    <t>Design of Prototype Readout Electronics of the High Counting Rate Main Drift Chamber in Particle Physics Experiments</t>
-  </si>
-  <si>
-    <t>Prototype Readout Electronics System for a LET Spectrometer in Space Radiation</t>
-  </si>
-  <si>
-    <t>A Full on-Chip LDO Regulator with self-adapting compensation networks for Front-end Readout Circuit</t>
-  </si>
-  <si>
-    <t>The μMUX readout electronic system of the AliCPT</t>
-  </si>
-  <si>
-    <t>Low-Noise Room-Temperature Readout Electronics for TDM-SQUID TES Arrays in the AliCPT-40G Telescope</t>
-  </si>
-  <si>
-    <t>A 14-bit 100 Ms/s Pipeline ADC for Silicon Pixel Sensor in Gaseous Detectors</t>
-  </si>
-  <si>
-    <t>Performance Test of the SAMIDARE Board with Mini-TPC using heavy-Ion Beams</t>
-  </si>
-  <si>
-    <t>Design of a Novel Pipelined SAR ADC for Multi-channel Front-end ASICs</t>
-  </si>
-  <si>
-    <t>Georg</t>
-  </si>
-  <si>
-    <t>Fernando</t>
-  </si>
-  <si>
-    <t>Kai</t>
-  </si>
-  <si>
-    <t>Dingjun</t>
-  </si>
-  <si>
-    <t>Yilin</t>
-  </si>
-  <si>
-    <t>Wenrui</t>
-  </si>
-  <si>
-    <t>xiayu</t>
-  </si>
-  <si>
-    <t>Xiangxiang</t>
-  </si>
-  <si>
-    <t>Tangchong</t>
-  </si>
-  <si>
-    <t>Haoqing</t>
-  </si>
-  <si>
-    <t>Fumitaka</t>
-  </si>
-  <si>
-    <t>Schardt</t>
-  </si>
-  <si>
-    <t>Carrio Argos</t>
-  </si>
-  <si>
-    <t>Shi</t>
-  </si>
-  <si>
-    <t>Ma</t>
-  </si>
-  <si>
-    <t>Sun</t>
-  </si>
-  <si>
-    <t>wang</t>
-  </si>
-  <si>
-    <t>Ren</t>
-  </si>
-  <si>
-    <t>Kuang</t>
-  </si>
-  <si>
-    <t>ENDO</t>
+    <t>Endo</t>
   </si>
   <si>
     <t>ITE</t>
@@ -1220,13 +1265,13 @@
     <t>Yimou</t>
   </si>
   <si>
-    <t>xin</t>
+    <t>Xin</t>
   </si>
   <si>
     <t>Carlos</t>
   </si>
   <si>
-    <t>A.</t>
+    <t>Anh</t>
   </si>
   <si>
     <t>Carlo</t>
@@ -1262,7 +1307,7 @@
     <t>Xiang</t>
   </si>
   <si>
-    <t>cao</t>
+    <t>Cao</t>
   </si>
   <si>
     <t>Abellan Beteta</t>
@@ -1310,9 +1355,6 @@
     <t>University of Zurich (CH)</t>
   </si>
   <si>
-    <t>Flerov Laboratory of Nuclear Reactions, JINR, 141980 Dubna, Russia</t>
-  </si>
-  <si>
     <t>Università di Pisa</t>
   </si>
   <si>
@@ -1343,9 +1385,6 @@
     <t>La Biodola</t>
   </si>
   <si>
-    <t>2025-05-25 14:45:00</t>
-  </si>
-  <si>
     <t>pi5pm1</t>
   </si>
   <si>
@@ -1428,42 +1467,6 @@
   </si>
   <si>
     <t>pi5pm28</t>
-  </si>
-  <si>
-    <t>Emerging Technologies, New Standards, Feedback on Experience &amp; Industry</t>
-  </si>
-  <si>
-    <t>AI, Machine Learning, Real Time Simulation, Intelligent Signal Processing</t>
-  </si>
-  <si>
-    <t>Real Time Diagnostics, Digital Twin, Control, Monitoring, Safety and Security - B</t>
-  </si>
-  <si>
-    <t>Front-End Electronics, Fast Digitizers, Fast Transfer Links &amp; Networks - A</t>
-  </si>
-  <si>
-    <t>Data Acquisition and Trigger Architectures - A</t>
-  </si>
-  <si>
-    <t>Real Time Diagnostics, Digital Twin, Control, Monitoring, Safety and Security - A</t>
-  </si>
-  <si>
-    <t>Front-End Electronics, Fast Digitizers, Fast Transfer Links &amp; Networks - B</t>
-  </si>
-  <si>
-    <t>Data Acquisition and Trigger Architectures - B</t>
-  </si>
-  <si>
-    <t>2026-05-16 16:20:00</t>
-  </si>
-  <si>
-    <t>2026-05-16 16:30:00</t>
-  </si>
-  <si>
-    <t>2026-05-16 16:25:00</t>
-  </si>
-  <si>
-    <t>2026-05-16 16:35:00</t>
   </si>
 </sst>
 </file>
@@ -1479,7 +1482,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1507,7 +1511,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1832,7 +1836,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>435</v>
+        <v>449</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1840,7 +1844,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>436</v>
+        <v>450</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1877,282 +1881,282 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>62</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>335</v>
+        <v>351</v>
       </c>
       <c r="D2" t="s">
-        <v>348</v>
+        <v>364</v>
       </c>
       <c r="E2" t="s">
-        <v>359</v>
+        <v>375</v>
       </c>
       <c r="F2" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>152</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>336</v>
+        <v>352</v>
       </c>
       <c r="D3" t="s">
-        <v>349</v>
+        <v>365</v>
       </c>
       <c r="E3" t="s">
-        <v>360</v>
+        <v>376</v>
       </c>
       <c r="F3" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>162</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>337</v>
+        <v>353</v>
       </c>
       <c r="D4" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="E4" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="F4" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>166</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="D5" t="s">
-        <v>350</v>
+        <v>366</v>
       </c>
       <c r="E5" t="s">
-        <v>361</v>
+        <v>377</v>
       </c>
       <c r="F5" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>178</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>339</v>
+        <v>355</v>
       </c>
       <c r="D6" t="s">
-        <v>351</v>
+        <v>367</v>
       </c>
       <c r="E6" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="F6" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>179</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>340</v>
+        <v>356</v>
       </c>
       <c r="D7" t="s">
-        <v>352</v>
+        <v>368</v>
       </c>
       <c r="E7" t="s">
-        <v>362</v>
+        <v>243</v>
       </c>
       <c r="F7" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>180</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>341</v>
+        <v>357</v>
       </c>
       <c r="D8" t="s">
-        <v>353</v>
+        <v>369</v>
       </c>
       <c r="E8" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="F8" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>181</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>342</v>
+        <v>358</v>
       </c>
       <c r="D9" t="s">
-        <v>354</v>
+        <v>370</v>
       </c>
       <c r="E9" t="s">
-        <v>364</v>
+        <v>130</v>
       </c>
       <c r="F9" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>182</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>343</v>
+        <v>359</v>
       </c>
       <c r="D10" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="E10" t="s">
-        <v>365</v>
+        <v>379</v>
       </c>
       <c r="F10" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>185</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="D11" t="s">
-        <v>356</v>
+        <v>372</v>
       </c>
       <c r="E11" t="s">
-        <v>366</v>
+        <v>380</v>
       </c>
       <c r="F11" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>190</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
       <c r="D12" t="s">
-        <v>357</v>
+        <v>373</v>
       </c>
       <c r="E12" t="s">
-        <v>220</v>
+        <v>381</v>
       </c>
       <c r="F12" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>194</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="D13" t="s">
-        <v>358</v>
+        <v>374</v>
       </c>
       <c r="E13" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="F13" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>200</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>347</v>
+        <v>363</v>
       </c>
       <c r="D14" t="s">
-        <v>357</v>
+        <v>373</v>
       </c>
       <c r="E14" t="s">
-        <v>220</v>
+        <v>381</v>
       </c>
       <c r="F14" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -2173,22 +2177,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -2199,16 +2203,16 @@
         <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
       <c r="D2" t="s">
-        <v>391</v>
+        <v>406</v>
       </c>
       <c r="E2" t="s">
-        <v>407</v>
+        <v>422</v>
       </c>
       <c r="F2" t="s">
-        <v>420</v>
+        <v>435</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -2219,16 +2223,16 @@
         <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
       <c r="D3" t="s">
-        <v>392</v>
+        <v>407</v>
       </c>
       <c r="E3" t="s">
-        <v>408</v>
+        <v>423</v>
       </c>
       <c r="F3" t="s">
-        <v>421</v>
+        <v>436</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -2239,16 +2243,16 @@
         <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="D4" t="s">
-        <v>393</v>
+        <v>408</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="F4" t="s">
-        <v>422</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -2259,16 +2263,16 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
       <c r="D5" t="s">
-        <v>394</v>
+        <v>409</v>
       </c>
       <c r="E5" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="F5" t="s">
-        <v>423</v>
+        <v>438</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -2279,16 +2283,16 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>377</v>
+        <v>392</v>
       </c>
       <c r="D6" t="s">
-        <v>395</v>
+        <v>410</v>
       </c>
       <c r="E6" t="s">
-        <v>409</v>
+        <v>424</v>
       </c>
       <c r="F6" t="s">
-        <v>424</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -2299,16 +2303,16 @@
         <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
       <c r="D7" t="s">
-        <v>396</v>
+        <v>411</v>
       </c>
       <c r="E7" t="s">
-        <v>410</v>
+        <v>425</v>
       </c>
       <c r="F7" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -2319,16 +2323,16 @@
         <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>379</v>
+        <v>394</v>
       </c>
       <c r="D8" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="E8" t="s">
-        <v>411</v>
+        <v>426</v>
       </c>
       <c r="F8" t="s">
-        <v>425</v>
+        <v>440</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -2339,16 +2343,13 @@
         <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="D9" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E9" t="s">
-        <v>412</v>
-      </c>
-      <c r="F9" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -2359,16 +2360,16 @@
         <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>381</v>
+        <v>396</v>
       </c>
       <c r="D10" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="E10" t="s">
-        <v>413</v>
+        <v>428</v>
       </c>
       <c r="F10" t="s">
-        <v>427</v>
+        <v>441</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -2379,16 +2380,16 @@
         <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>382</v>
+        <v>397</v>
       </c>
       <c r="D11" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="E11" t="s">
-        <v>414</v>
+        <v>429</v>
       </c>
       <c r="F11" t="s">
-        <v>428</v>
+        <v>442</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -2399,16 +2400,16 @@
         <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>383</v>
+        <v>398</v>
       </c>
       <c r="D12" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="E12" t="s">
-        <v>415</v>
+        <v>430</v>
       </c>
       <c r="F12" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -2419,16 +2420,16 @@
         <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
       <c r="D13" t="s">
-        <v>401</v>
+        <v>416</v>
       </c>
       <c r="E13" t="s">
-        <v>416</v>
+        <v>431</v>
       </c>
       <c r="F13" t="s">
-        <v>429</v>
+        <v>443</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -2439,16 +2440,16 @@
         <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="D14" t="s">
-        <v>402</v>
+        <v>417</v>
       </c>
       <c r="E14" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="F14" t="s">
-        <v>430</v>
+        <v>444</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -2459,16 +2460,16 @@
         <v>26</v>
       </c>
       <c r="C15" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
       <c r="D15" t="s">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="F15" t="s">
-        <v>431</v>
+        <v>445</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -2479,16 +2480,16 @@
         <v>27</v>
       </c>
       <c r="C16" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
       <c r="D16" t="s">
-        <v>404</v>
+        <v>419</v>
       </c>
       <c r="E16" t="s">
-        <v>417</v>
+        <v>432</v>
       </c>
       <c r="F16" t="s">
-        <v>432</v>
+        <v>446</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -2499,16 +2500,16 @@
         <v>28</v>
       </c>
       <c r="C17" t="s">
-        <v>388</v>
+        <v>403</v>
       </c>
       <c r="D17" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="E17" t="s">
-        <v>220</v>
+        <v>381</v>
       </c>
       <c r="F17" t="s">
-        <v>433</v>
+        <v>447</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -2519,16 +2520,16 @@
         <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>389</v>
+        <v>404</v>
       </c>
       <c r="D18" t="s">
-        <v>405</v>
+        <v>420</v>
       </c>
       <c r="E18" t="s">
-        <v>418</v>
+        <v>433</v>
       </c>
       <c r="F18" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -2539,16 +2540,16 @@
         <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="D19" t="s">
-        <v>406</v>
+        <v>421</v>
       </c>
       <c r="E19" t="s">
-        <v>419</v>
+        <v>434</v>
       </c>
       <c r="F19" t="s">
-        <v>434</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>
@@ -2585,13 +2586,13 @@
         <v>28931</v>
       </c>
       <c r="B2" t="s">
-        <v>466</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>474</v>
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -2599,13 +2600,13 @@
         <v>28932</v>
       </c>
       <c r="B3" t="s">
-        <v>469</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>474</v>
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -2613,13 +2614,13 @@
         <v>28933</v>
       </c>
       <c r="B4" t="s">
-        <v>467</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>476</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>475</v>
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -2627,13 +2628,13 @@
         <v>28934</v>
       </c>
       <c r="B5" t="s">
-        <v>468</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>476</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>475</v>
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -2641,13 +2642,13 @@
         <v>28935</v>
       </c>
       <c r="B6" t="s">
-        <v>470</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>476</v>
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -2655,13 +2656,13 @@
         <v>28936</v>
       </c>
       <c r="B7" t="s">
-        <v>471</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>476</v>
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -2669,13 +2670,13 @@
         <v>28937</v>
       </c>
       <c r="B8" t="s">
-        <v>472</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>477</v>
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -2683,17 +2684,16 @@
         <v>28938</v>
       </c>
       <c r="B9" t="s">
-        <v>473</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>477</v>
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2708,15 +2708,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>438</v>
+        <v>451</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2724,7 +2724,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>439</v>
+        <v>452</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -2732,7 +2732,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>440</v>
+        <v>453</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -2740,7 +2740,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>441</v>
+        <v>454</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -2748,7 +2748,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>442</v>
+        <v>455</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -2756,7 +2756,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>443</v>
+        <v>456</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -2764,7 +2764,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>444</v>
+        <v>457</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -2772,7 +2772,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>445</v>
+        <v>458</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -2780,7 +2780,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>446</v>
+        <v>459</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -2788,7 +2788,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>447</v>
+        <v>460</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -2796,7 +2796,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>448</v>
+        <v>461</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -2804,7 +2804,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>449</v>
+        <v>462</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -2812,7 +2812,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>450</v>
+        <v>463</v>
       </c>
       <c r="B14">
         <v>13</v>
@@ -2820,7 +2820,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>451</v>
+        <v>464</v>
       </c>
       <c r="B15">
         <v>14</v>
@@ -2828,7 +2828,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>452</v>
+        <v>465</v>
       </c>
       <c r="B16">
         <v>15</v>
@@ -2836,7 +2836,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="B17">
         <v>16</v>
@@ -2844,7 +2844,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="B18">
         <v>17</v>
@@ -2852,7 +2852,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>455</v>
+        <v>468</v>
       </c>
       <c r="B19">
         <v>18</v>
@@ -2860,7 +2860,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>456</v>
+        <v>469</v>
       </c>
       <c r="B20">
         <v>19</v>
@@ -2868,7 +2868,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>457</v>
+        <v>470</v>
       </c>
       <c r="B21">
         <v>20</v>
@@ -2876,7 +2876,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>458</v>
+        <v>471</v>
       </c>
       <c r="B22">
         <v>21</v>
@@ -2884,7 +2884,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>459</v>
+        <v>472</v>
       </c>
       <c r="B23">
         <v>22</v>
@@ -2892,7 +2892,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>460</v>
+        <v>473</v>
       </c>
       <c r="B24">
         <v>23</v>
@@ -2900,7 +2900,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>461</v>
+        <v>474</v>
       </c>
       <c r="B25">
         <v>24</v>
@@ -2908,7 +2908,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>462</v>
+        <v>475</v>
       </c>
       <c r="B26">
         <v>25</v>
@@ -2916,7 +2916,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>463</v>
+        <v>476</v>
       </c>
       <c r="B27">
         <v>26</v>
@@ -2924,7 +2924,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>464</v>
+        <v>477</v>
       </c>
       <c r="B28">
         <v>27</v>
@@ -2932,7 +2932,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>465</v>
+        <v>478</v>
       </c>
       <c r="B29">
         <v>28</v>
@@ -2956,22 +2956,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -2982,16 +2982,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -3002,13 +3002,16 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>48</v>
+      </c>
+      <c r="F3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -3019,16 +3022,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -3039,16 +3042,16 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -3059,13 +3062,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>51</v>
+      </c>
+      <c r="F6" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -3076,16 +3082,16 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -3106,22 +3112,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -3132,16 +3138,16 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="E2" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="F2" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -3152,16 +3158,16 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="E3" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="F3" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -3172,16 +3178,16 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E4" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="F4" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -3192,16 +3198,16 @@
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="F5" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -3212,16 +3218,16 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="E6" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="F6" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -3232,16 +3238,16 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="E7" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="F7" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -3252,16 +3258,16 @@
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="D8" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="E8" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="F8" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -3272,16 +3278,16 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="D9" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="E9" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="F9" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -3292,16 +3298,16 @@
         <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="F10" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -3312,16 +3318,16 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="E11" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="F11" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -3332,16 +3338,16 @@
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="E12" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="F12" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -3352,16 +3358,16 @@
         <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D13" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="F13" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -3372,16 +3378,16 @@
         <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="E14" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="F14" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -3392,16 +3398,16 @@
         <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="E15" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="F15" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -3412,16 +3418,16 @@
         <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="E16" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="F16" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -3432,13 +3438,16 @@
         <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="E17" t="s">
-        <v>108</v>
+        <v>126</v>
+      </c>
+      <c r="F17" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -3449,16 +3458,16 @@
         <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="D18" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="E18" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="F18" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -3469,13 +3478,13 @@
         <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="D19" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="E19" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -3486,13 +3495,13 @@
         <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="E20" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -3503,16 +3512,16 @@
         <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="E21" t="s">
-        <v>111</v>
+        <v>129</v>
       </c>
       <c r="F21" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -3523,16 +3532,16 @@
         <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="D22" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="E22" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="F22" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -3543,16 +3552,16 @@
         <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="D23" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="E23" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="F23" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -3563,16 +3572,16 @@
         <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="D24" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="E24" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="F24" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -3583,16 +3592,16 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="D25" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="E25" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="F25" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -3603,16 +3612,16 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="E26" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="F26" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -3623,16 +3632,16 @@
         <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D27" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="E27" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="F27" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -3643,16 +3652,16 @@
         <v>18</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="D28" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="E28" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="F28" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -3673,22 +3682,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -3699,16 +3708,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="D2" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="E2" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="F2" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -3719,16 +3728,16 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="D3" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="E3" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="F3" t="s">
-        <v>179</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -3739,16 +3748,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
       <c r="E4" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="F4" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -3759,16 +3768,16 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="D5" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="E5" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="F5" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -3779,16 +3788,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="D6" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="E6" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="F6" t="s">
-        <v>180</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -3799,16 +3808,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="E7" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="F7" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -3819,16 +3828,16 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="D8" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="E8" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="F8" t="s">
-        <v>181</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -3839,16 +3848,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="D9" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
       <c r="E9" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="F9" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -3859,13 +3868,16 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="E10" t="s">
-        <v>172</v>
+        <v>190</v>
+      </c>
+      <c r="F10" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -3876,13 +3888,16 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="D11" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="E11" t="s">
-        <v>173</v>
+        <v>191</v>
+      </c>
+      <c r="F11" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -3893,16 +3908,16 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="D12" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="E12" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
       <c r="F12" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -3913,16 +3928,16 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="D13" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="E13" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="F13" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -3933,13 +3948,13 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="D14" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="E14" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -3950,13 +3965,16 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="D15" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="E15" t="s">
-        <v>176</v>
+        <v>194</v>
+      </c>
+      <c r="F15" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -3967,13 +3985,13 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
       <c r="D16" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="E16" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -3984,13 +4002,13 @@
         <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="D17" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="E17" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -4011,22 +4029,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -4037,16 +4055,16 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>185</v>
+        <v>206</v>
       </c>
       <c r="D2" t="s">
-        <v>202</v>
+        <v>223</v>
       </c>
       <c r="E2" t="s">
-        <v>217</v>
+        <v>237</v>
       </c>
       <c r="F2" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4057,16 +4075,16 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="D3" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="E3" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="F3" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -4077,16 +4095,16 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
       <c r="D4" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
       <c r="E4" t="s">
-        <v>218</v>
+        <v>238</v>
       </c>
       <c r="F4" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4097,13 +4115,16 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="D5" t="s">
-        <v>204</v>
+        <v>225</v>
       </c>
       <c r="E5" t="s">
-        <v>219</v>
+        <v>239</v>
+      </c>
+      <c r="F5" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -4114,16 +4135,16 @@
         <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
       <c r="D6" t="s">
-        <v>205</v>
+        <v>226</v>
       </c>
       <c r="E6" t="s">
-        <v>220</v>
+        <v>134</v>
       </c>
       <c r="F6" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -4134,16 +4155,16 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="D7" t="s">
-        <v>206</v>
+        <v>227</v>
       </c>
       <c r="E7" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="F7" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -4154,16 +4175,16 @@
         <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="D8" t="s">
-        <v>207</v>
+        <v>228</v>
       </c>
       <c r="E8" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
       <c r="F8" t="s">
-        <v>234</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -4174,13 +4195,16 @@
         <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="D9" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="E9" t="s">
-        <v>223</v>
+        <v>242</v>
+      </c>
+      <c r="F9" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -4191,16 +4215,16 @@
         <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>193</v>
+        <v>214</v>
       </c>
       <c r="D10" t="s">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="E10" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="F10" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -4211,16 +4235,16 @@
         <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
       <c r="D11" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="E11" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="F11" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -4231,16 +4255,16 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="D12" t="s">
-        <v>211</v>
+        <v>231</v>
       </c>
       <c r="E12" t="s">
-        <v>225</v>
+        <v>243</v>
       </c>
       <c r="F12" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -4251,16 +4275,16 @@
         <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="D13" t="s">
-        <v>212</v>
+        <v>232</v>
       </c>
       <c r="E13" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="F13" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -4271,16 +4295,16 @@
         <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="D14" t="s">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="E14" t="s">
-        <v>226</v>
+        <v>244</v>
       </c>
       <c r="F14" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -4291,16 +4315,16 @@
         <v>28</v>
       </c>
       <c r="C15" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="D15" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
       <c r="E15" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="F15" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -4311,13 +4335,16 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="D16" t="s">
-        <v>215</v>
+        <v>235</v>
       </c>
       <c r="E16" t="s">
-        <v>227</v>
+        <v>245</v>
+      </c>
+      <c r="F16" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -4328,16 +4355,16 @@
         <v>19</v>
       </c>
       <c r="C17" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="D17" t="s">
-        <v>216</v>
+        <v>236</v>
       </c>
       <c r="E17" t="s">
-        <v>228</v>
+        <v>246</v>
       </c>
       <c r="F17" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -4348,16 +4375,16 @@
         <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="E18" t="s">
-        <v>229</v>
+        <v>247</v>
       </c>
       <c r="F18" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -4367,7 +4394,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12.6640625" customWidth="1"/>
@@ -4378,290 +4405,282 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
       <c r="D2" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
       <c r="E2" t="s">
-        <v>266</v>
+        <v>126</v>
       </c>
       <c r="F2" t="s">
-        <v>277</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
       <c r="D3" t="s">
-        <v>254</v>
+        <v>89</v>
       </c>
       <c r="E3" t="s">
-        <v>108</v>
+        <v>281</v>
       </c>
       <c r="F3" t="s">
-        <v>118</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
       <c r="D4" t="s">
-        <v>255</v>
+        <v>272</v>
       </c>
       <c r="E4" t="s">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="F4" t="s">
-        <v>278</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="D5" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
       <c r="E5" t="s">
-        <v>268</v>
+        <v>283</v>
+      </c>
+      <c r="F5" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
       <c r="D6" t="s">
-        <v>257</v>
+        <v>86</v>
       </c>
       <c r="E6" t="s">
-        <v>269</v>
+        <v>284</v>
       </c>
       <c r="F6" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="D7" t="s">
-        <v>68</v>
+        <v>274</v>
       </c>
       <c r="E7" t="s">
-        <v>270</v>
+        <v>285</v>
+      </c>
+      <c r="F7" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="D8" t="s">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="E8" t="s">
-        <v>271</v>
+        <v>116</v>
+      </c>
+      <c r="F8" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="D9" t="s">
-        <v>259</v>
+        <v>276</v>
       </c>
       <c r="E9" t="s">
-        <v>98</v>
+        <v>286</v>
+      </c>
+      <c r="F9" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B10">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
       <c r="D10" t="s">
-        <v>260</v>
+        <v>277</v>
       </c>
       <c r="E10" t="s">
-        <v>272</v>
+        <v>287</v>
       </c>
       <c r="F10" t="s">
-        <v>280</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B11">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="D11" t="s">
-        <v>261</v>
+        <v>115</v>
       </c>
       <c r="E11" t="s">
-        <v>273</v>
+        <v>120</v>
       </c>
       <c r="F11" t="s">
-        <v>281</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="B12">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
       <c r="D12" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
       <c r="E12" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="F12" t="s">
-        <v>282</v>
+        <v>298</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B13">
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>250</v>
+        <v>269</v>
       </c>
       <c r="D13" t="s">
-        <v>263</v>
+        <v>279</v>
       </c>
       <c r="E13" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="F13" t="s">
-        <v>283</v>
+        <v>299</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="B14">
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
       <c r="D14" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="E14" t="s">
-        <v>276</v>
+        <v>120</v>
       </c>
       <c r="F14" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>126</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15" t="s">
-        <v>252</v>
-      </c>
-      <c r="D15" t="s">
-        <v>265</v>
-      </c>
-      <c r="E15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F15" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -4682,22 +4701,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -4708,16 +4727,16 @@
         <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>285</v>
+        <v>300</v>
       </c>
       <c r="D2" t="s">
-        <v>301</v>
+        <v>316</v>
       </c>
       <c r="E2" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="F2" t="s">
-        <v>325</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4728,16 +4747,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>286</v>
+        <v>301</v>
       </c>
       <c r="D3" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="E3" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
       <c r="F3" t="s">
-        <v>326</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -4748,16 +4767,16 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>287</v>
+        <v>302</v>
       </c>
       <c r="D4" t="s">
-        <v>303</v>
+        <v>318</v>
       </c>
       <c r="E4" t="s">
-        <v>317</v>
+        <v>331</v>
       </c>
       <c r="F4" t="s">
-        <v>232</v>
+        <v>341</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4768,16 +4787,16 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="D5" t="s">
-        <v>304</v>
+        <v>319</v>
       </c>
       <c r="E5" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="F5" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -4788,16 +4807,16 @@
         <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>289</v>
+        <v>304</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
-        <v>318</v>
+        <v>332</v>
       </c>
       <c r="F6" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -4808,13 +4827,16 @@
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>290</v>
+        <v>305</v>
       </c>
       <c r="D7" t="s">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="E7" t="s">
-        <v>223</v>
+        <v>242</v>
+      </c>
+      <c r="F7" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -4825,16 +4847,16 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>291</v>
+        <v>306</v>
       </c>
       <c r="D8" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="E8" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="F8" t="s">
-        <v>284</v>
+        <v>299</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -4845,13 +4867,16 @@
         <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>292</v>
+        <v>307</v>
       </c>
       <c r="D9" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="E9" t="s">
-        <v>320</v>
+        <v>334</v>
+      </c>
+      <c r="F9" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -4862,16 +4887,16 @@
         <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>293</v>
+        <v>308</v>
       </c>
       <c r="D10" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
       <c r="E10" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
       <c r="F10" t="s">
-        <v>328</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -4882,16 +4907,16 @@
         <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="D11" t="s">
-        <v>309</v>
+        <v>324</v>
       </c>
       <c r="E11" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="F11" t="s">
-        <v>329</v>
+        <v>346</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -4902,16 +4927,16 @@
         <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>295</v>
+        <v>310</v>
       </c>
       <c r="D12" t="s">
-        <v>264</v>
+        <v>279</v>
       </c>
       <c r="E12" t="s">
-        <v>322</v>
+        <v>336</v>
       </c>
       <c r="F12" t="s">
-        <v>330</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -4922,16 +4947,16 @@
         <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>296</v>
+        <v>311</v>
       </c>
       <c r="D13" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="E13" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="F13" t="s">
-        <v>331</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -4942,16 +4967,16 @@
         <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>297</v>
+        <v>312</v>
       </c>
       <c r="D14" t="s">
-        <v>311</v>
+        <v>326</v>
       </c>
       <c r="E14" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="F14" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -4962,16 +4987,16 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>298</v>
+        <v>313</v>
       </c>
       <c r="D15" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E15" t="s">
-        <v>323</v>
+        <v>337</v>
       </c>
       <c r="F15" t="s">
-        <v>333</v>
+        <v>349</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -4982,13 +5007,16 @@
         <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>299</v>
+        <v>314</v>
       </c>
       <c r="D16" t="s">
-        <v>313</v>
+        <v>226</v>
       </c>
       <c r="E16" t="s">
-        <v>116</v>
+        <v>134</v>
+      </c>
+      <c r="F16" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -4999,16 +5027,16 @@
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>300</v>
+        <v>315</v>
       </c>
       <c r="D17" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
       <c r="E17" t="s">
-        <v>324</v>
+        <v>338</v>
       </c>
       <c r="F17" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
revised program and new posters
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marco/work/git/rt2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{747DC37F-FA9B-DF42-91F6-1FDB1DABFD27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777811DD-CEAF-9F41-904F-F629C2BC3F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="14680" windowHeight="17160" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="600" windowWidth="25260" windowHeight="26880" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="447">
   <si>
     <t>Key</t>
   </si>
@@ -152,9 +152,6 @@
     <t>EJFAT - ESnet / Jefferson Lab FPGA Accelerated Transport.  Design Improvements and User Experiences.</t>
   </si>
   <si>
-    <t>An FPGA-based Streaming DAQ emulator for evaluating and tuning DAQ networks and data management infrastruc-ture.</t>
-  </si>
-  <si>
     <t>Stefano</t>
   </si>
   <si>
@@ -170,9 +167,6 @@
     <t>Yatish</t>
   </si>
   <si>
-    <t>Jeff</t>
-  </si>
-  <si>
     <t>Pavinato</t>
   </si>
   <si>
@@ -188,16 +182,13 @@
     <t>Kumar</t>
   </si>
   <si>
-    <t>Maggio</t>
-  </si>
-  <si>
     <t>European Spallation Source</t>
   </si>
   <si>
     <t>KIT</t>
   </si>
   <si>
-    <t>Science and Technology Facilities Council STFC (GB)</t>
+    <t>Science and Technology Facilities Council</t>
   </si>
   <si>
     <t>Max-Planck-Institute for Plasma Physics</t>
@@ -206,9 +197,6 @@
     <t>Energy Sciences Network</t>
   </si>
   <si>
-    <t>SkuTek Instrumentation</t>
-  </si>
-  <si>
     <t>Performance evaluation of ITER Synchronous Data Network using Time Sensitive Network</t>
   </si>
   <si>
@@ -236,7 +224,7 @@
     <t>Tapped Delay Lines Time-to-digital converter design and performance in Versal architecture</t>
   </si>
   <si>
-    <t>Progress in Readout Electronics for Scintillator-Based Multi-Neutron Detector Array</t>
+    <t>Design of the Readout Electronics for Scintillator-Based Multi-Neutron Detector Array</t>
   </si>
   <si>
     <t>Extension of a wired time-synchronization protocol for sub-nanosecond accuracy to multiple FPGA families</t>
@@ -329,7 +317,7 @@
     <t>Qingkang</t>
   </si>
   <si>
-    <t>jiayun</t>
+    <t>Jiayun</t>
   </si>
   <si>
     <t>Chunlai</t>
@@ -407,9 +395,6 @@
     <t>Wu</t>
   </si>
   <si>
-    <t>chen</t>
-  </si>
-  <si>
     <t>Dong</t>
   </si>
   <si>
@@ -449,13 +434,10 @@
     <t>KEK</t>
   </si>
   <si>
-    <t>University of Science and  Technology of China (CN)</t>
-  </si>
-  <si>
-    <t>the Department of Modern Physics, University of Science and Technology of China, Hefei 230026, China</t>
-  </si>
-  <si>
-    <t>Department of Modern Physics, University of Science and Technology of China</t>
+    <t>University of Science and  Technology of China</t>
+  </si>
+  <si>
+    <t>University of Science and Technology of China, Hefei</t>
   </si>
   <si>
     <t>University of California, Davis</t>
@@ -470,330 +452,303 @@
     <t>Nanjing University,  IHEP</t>
   </si>
   <si>
-    <t>山东大学</t>
-  </si>
-  <si>
     <t>Central China Normal University</t>
   </si>
   <si>
     <t>CAEN S.p.A.</t>
   </si>
   <si>
+    <t>IHEP, Chinese Academy of Sciences</t>
+  </si>
+  <si>
+    <t>Nanjing University</t>
+  </si>
+  <si>
+    <t>RIKEN Nishina Center</t>
+  </si>
+  <si>
+    <t>Institute of High Energy Physics</t>
+  </si>
+  <si>
+    <t>FPGA-Deployed Variational Autoencoder for Real-Time Soft X-Ray Electron Temperature Reconstruction in RFX-mod2</t>
+  </si>
+  <si>
+    <t>Design-Space Exploration and Integer Quantization of Graph Neural Networks for Real-Time FPGA Track Finding</t>
+  </si>
+  <si>
+    <t>An Initial Study of Neural-Network-Assisted Approaches for Drift Chamber Tracking</t>
+  </si>
+  <si>
+    <t>Real-time Autoregressive Evolution of Tokamak Plasma Magnetic Measurements</t>
+  </si>
+  <si>
+    <t>A High-performance DOI Encoding Algorithm for PET Detectors with High Coupling Ratio</t>
+  </si>
+  <si>
+    <t>Real-Time Machine-Learning Inference Workflows at FRIB using EJFAT and ESNet</t>
+  </si>
+  <si>
+    <t>Event-Driven Spiking Neural Networks for Emergent Robotic Swarm Behavior</t>
+  </si>
+  <si>
+    <t>A Maximum Log-Likelihood Regression Approach for Quantitative Mixture Prediction in PGNAA Spectroscopy</t>
+  </si>
+  <si>
+    <t>Studies for a track finder algorithm based on Graph Neural Networks for the MEG II experiment</t>
+  </si>
+  <si>
+    <t>A Scalable Intelligent Agent System for Automated Monitoring and Debugging Support of the JUNO Electronics system</t>
+  </si>
+  <si>
+    <t>Real-Time Plasma Density Prediction and Control Framework for Pellet Injection on EAST Tokamak</t>
+  </si>
+  <si>
+    <t>A 1D-Convolutional Autoencoder for Pulse Compression in Nuclear DAQ Systems</t>
+  </si>
+  <si>
+    <t>Single-Detector Cosmic-Ray Muon Identification in Plastic Scintillators Using Machine Learning</t>
+  </si>
+  <si>
+    <t>Self-Supervised and Semi-Supervised Machine Learning for Waveform-Based Neutron/Gamma Discrimination in EJ-276 Plastic Scintillator</t>
+  </si>
+  <si>
+    <t>Luca</t>
+  </si>
+  <si>
+    <t>Andrea</t>
+  </si>
+  <si>
+    <t>Viet</t>
+  </si>
+  <si>
+    <t>Shuai</t>
+  </si>
+  <si>
+    <t>Yonggang</t>
+  </si>
+  <si>
+    <t>Giordano</t>
+  </si>
+  <si>
+    <t>Marcos</t>
+  </si>
+  <si>
+    <t>Helmand</t>
+  </si>
+  <si>
+    <t>Antoine</t>
+  </si>
+  <si>
+    <t>Yifan</t>
+  </si>
+  <si>
+    <t>Yucheng</t>
+  </si>
+  <si>
+    <t>Jose  Manuel</t>
+  </si>
+  <si>
+    <t>Hai</t>
+  </si>
+  <si>
+    <t>Orlandi</t>
+  </si>
+  <si>
+    <t>Cardini</t>
+  </si>
+  <si>
+    <t>Nguyen</t>
+  </si>
+  <si>
+    <t>Cerizza</t>
+  </si>
+  <si>
+    <t>Turqueti</t>
+  </si>
+  <si>
+    <t>Shayan</t>
+  </si>
+  <si>
+    <t>Venturini</t>
+  </si>
+  <si>
+    <t>Yang</t>
+  </si>
+  <si>
+    <t>Deltoro  Berrio</t>
+  </si>
+  <si>
+    <t>Vo</t>
+  </si>
+  <si>
+    <t>Università di Padova - Consorzio RFX</t>
+  </si>
+  <si>
+    <t>Universidad de Oviedo</t>
+  </si>
+  <si>
+    <t>Institute of Energy, Hefei</t>
+  </si>
+  <si>
+    <t>Facility for Rare Isotope Beams @ Michigan State University</t>
+  </si>
+  <si>
+    <t>Lawrence Berkley National Laboratory</t>
+  </si>
+  <si>
+    <t>Technische Hochschule Ostwestfalen</t>
+  </si>
+  <si>
+    <t>INFN Pisa</t>
+  </si>
+  <si>
+    <t>Institute of Plasma Physics,Chinese Academy of Sciences</t>
+  </si>
+  <si>
+    <t>Universitat de València</t>
+  </si>
+  <si>
+    <t>A Low-Latency Distributed Machine-Protection System for the PIP-II Linear Accelerator</t>
+  </si>
+  <si>
+    <t>Temperature-Induced Delay Drift in Xilinx FPGA Multi-gigabit Transceivers</t>
+  </si>
+  <si>
+    <t>Deep Learning–Based Real-Time Error Detection in Radiotherapy with EPID Images</t>
+  </si>
+  <si>
+    <t>High-dose-rate precise ionization chamber with real-time electronics for SC cyclotron-based proton therapy system</t>
+  </si>
+  <si>
+    <t>Realization of Large Model-Driven Tango Control and Data Interaction Analysis Tool</t>
+  </si>
+  <si>
+    <t>A Virtual Gamma-ray Spectrum Database for Training in Seawater Radioactivity Analysis</t>
+  </si>
+  <si>
+    <t>Optimising SiPM Array Architectures and Optical Coatings for High-Efficiency ZnSe(Al,O)–Based Strontium-90 Detection</t>
+  </si>
+  <si>
+    <t>Ion Irradiation facility with Performance Online Monitoring for High Temperature Superconducting Tape</t>
+  </si>
+  <si>
+    <t>The Realization of Ultra-High Dose Rate and Potential Frontier Applications on 230 MeV SC Cyclotron CYCIAE-230</t>
+  </si>
+  <si>
+    <t>AI Enhanced LLRF Controller for Ultra-lightweight SC Cyclotron CYCIAE-100B</t>
+  </si>
+  <si>
+    <t>Design of an Integrated Control System for Automated Operation of  Large Array of Imaging Atmospheric Cherenkov Telescope</t>
+  </si>
+  <si>
+    <t>Physics-Aware and Hardware-Efficient Federated Learning for Isotope Identification in Distributed Edge Radiation Networks</t>
+  </si>
+  <si>
+    <t>Design and Implementation of a Space Radiation Microdosimetric Detection Prototype</t>
+  </si>
+  <si>
+    <t>Design of Transmission Cable Delay Calibration Method for Large-Scale Electron Accelerators</t>
+  </si>
+  <si>
+    <t>Application of the FPGA Coprocessor TM FAST for Siemens S7-1500 PLCs in Neutron Instruments</t>
+  </si>
+  <si>
+    <t>A common framework for real-time structured data communication in fusion devices</t>
+  </si>
+  <si>
+    <t>Fueling modeling and control for ITER start of research operation</t>
+  </si>
+  <si>
+    <t>Jonathan Daniel</t>
+  </si>
+  <si>
+    <t>Emmanuel</t>
+  </si>
+  <si>
+    <t>Tianyi</t>
+  </si>
+  <si>
+    <t>Huang</t>
+  </si>
+  <si>
+    <t>Wanook</t>
+  </si>
+  <si>
+    <t>Arjana</t>
+  </si>
+  <si>
+    <t>Xiaofeng</t>
+  </si>
+  <si>
+    <t>Tianjue</t>
+  </si>
+  <si>
+    <t>Si</t>
+  </si>
+  <si>
+    <t>Yuxin</t>
+  </si>
+  <si>
+    <t>Xiaoyan</t>
+  </si>
+  <si>
+    <t>Haoqian</t>
+  </si>
+  <si>
+    <t>Harald</t>
+  </si>
+  <si>
+    <t>Nicolo</t>
+  </si>
+  <si>
+    <t>Eisch</t>
+  </si>
+  <si>
+    <t>Uwitonze</t>
+  </si>
+  <si>
+    <t>Jiang</t>
+  </si>
+  <si>
+    <t>Ji</t>
+  </si>
+  <si>
+    <t>Kolnikaj</t>
+  </si>
+  <si>
+    <t>Zhu</t>
+  </si>
+  <si>
+    <t>Ma</t>
+  </si>
+  <si>
+    <t>Gao</t>
+  </si>
+  <si>
+    <t>Kleines</t>
+  </si>
+  <si>
+    <t>Ferron</t>
+  </si>
+  <si>
+    <t>Weldon</t>
+  </si>
+  <si>
+    <t>Fermi National Accelerator Lab.</t>
+  </si>
+  <si>
+    <t>China Institute of Atomic Energy</t>
+  </si>
+  <si>
+    <t>Korea Atomic Energy Research Institute</t>
+  </si>
+  <si>
+    <t>University of Glasgow</t>
+  </si>
+  <si>
     <t>Institute of High Energy Physics, Chinese Academy of Sciences</t>
   </si>
   <si>
-    <t>Nanjing University</t>
-  </si>
-  <si>
-    <t>RIKEN Nishina Center</t>
-  </si>
-  <si>
-    <t>Institute of High Energy Physics</t>
-  </si>
-  <si>
-    <t>FPGA-Deployed Variational Autoencoder for Real-Time Soft X-Ray Electron Temperature Reconstruction in RFX-mod2</t>
-  </si>
-  <si>
-    <t>Design-Space Exploration and Integer Quantization of Graph Neural Networks for Real-Time FPGA Track Finding</t>
-  </si>
-  <si>
-    <t>Intelligent Pulse Timing on Digitized Nuclear Signals with Self-Weakly-Supervised Neural Regression Models</t>
-  </si>
-  <si>
-    <t>An Initial Study of Neural-Network-Assisted Approaches for Drift Chamber Tracking</t>
-  </si>
-  <si>
-    <t>Real-time Autoregressive Evolution of Tokamak Plasma Magnetic Measurements</t>
-  </si>
-  <si>
-    <t>A High-performance DOI Encoding Algorithm for PET Detectors with High Coupling Ratio</t>
-  </si>
-  <si>
-    <t>Benchmarking Neural Network Inference on Versal ACAP AI Engines for Real-Time Detector Alignment</t>
-  </si>
-  <si>
-    <t>Real-Time Machine-Learning Inference Workflows at FRIB using EJFAT and ESNet</t>
-  </si>
-  <si>
-    <t>Event-Driven Spiking Neural Networks for Emergent Robotic Swarm Behavior</t>
-  </si>
-  <si>
-    <t>A Maximum Log-Likelihood Regression Approach for Quantitative Mixture Prediction in PGNAA Spectroscopy</t>
-  </si>
-  <si>
-    <t>Studies for a track finder algorithm based on Graph Neural Networks for the MEG II experiment</t>
-  </si>
-  <si>
-    <t>A Scalable Intelligent Agent System for Automated Monitoring and Debugging Support of the JUNO Electronics system</t>
-  </si>
-  <si>
-    <t>Real-Time Plasma Density Prediction and Control Framework for Pellet Injection on EAST Tokamak</t>
-  </si>
-  <si>
-    <t>A 1D-Convolutional Autoencoder for Pulse Compression in Nuclear DAQ Systems</t>
-  </si>
-  <si>
-    <t>Single-Detector Cosmic-Ray Muon Identification in Plastic Scintillators Using Machine Learning</t>
-  </si>
-  <si>
-    <t>Self-Supervised and Semi-Supervised Machine Learning for Waveform-Based Neutron/Gamma Discrimination in EJ-276 Plastic Scintillator</t>
-  </si>
-  <si>
-    <t>Luca</t>
-  </si>
-  <si>
-    <t>Andrea</t>
-  </si>
-  <si>
-    <t>Pengcheng</t>
-  </si>
-  <si>
-    <t>Viet</t>
-  </si>
-  <si>
-    <t>Shuai</t>
-  </si>
-  <si>
-    <t>Yonggang</t>
-  </si>
-  <si>
-    <t>Akshay</t>
-  </si>
-  <si>
-    <t>Giordano</t>
-  </si>
-  <si>
-    <t>Marcos</t>
-  </si>
-  <si>
-    <t>Helmand</t>
-  </si>
-  <si>
-    <t>Antoine</t>
-  </si>
-  <si>
-    <t>Yifan</t>
-  </si>
-  <si>
-    <t>Yucheng</t>
-  </si>
-  <si>
-    <t>Jose  Manuel</t>
-  </si>
-  <si>
-    <t>Hai</t>
-  </si>
-  <si>
-    <t>Orlandi</t>
-  </si>
-  <si>
-    <t>Cardini</t>
-  </si>
-  <si>
-    <t>Ai</t>
-  </si>
-  <si>
-    <t>Nguyen</t>
-  </si>
-  <si>
-    <t>Malige</t>
-  </si>
-  <si>
-    <t>Cerizza</t>
-  </si>
-  <si>
-    <t>Turqueti</t>
-  </si>
-  <si>
-    <t>Shayan</t>
-  </si>
-  <si>
-    <t>Venturini</t>
-  </si>
-  <si>
-    <t>Yang</t>
-  </si>
-  <si>
-    <t>Deltoro  Berrio</t>
-  </si>
-  <si>
-    <t>Vo</t>
-  </si>
-  <si>
-    <t>Università di Padova - Consorzio RFX</t>
-  </si>
-  <si>
-    <t>Universidad de Oviedo</t>
-  </si>
-  <si>
-    <t>Institute of Energy, Hefei Comprehensive National Science Center（Anhui Energy Laboratory)</t>
-  </si>
-  <si>
-    <t>Brookhaven National Laboratory (US)</t>
-  </si>
-  <si>
-    <t>Facility for Rare Isotope Beams @ Michigan State University</t>
-  </si>
-  <si>
-    <t>Lawrence Berkley National Laboratory</t>
-  </si>
-  <si>
-    <t>Technische Hochschule Ostwestfalen</t>
-  </si>
-  <si>
-    <t>INFN Pisa</t>
-  </si>
-  <si>
-    <t>Universite Libre de Bruxelles (BE)</t>
-  </si>
-  <si>
-    <t>Universitat de València</t>
-  </si>
-  <si>
-    <t>A Low-Latency Distributed Machine-Protection System for the PIP-II Linear Accelerator</t>
-  </si>
-  <si>
-    <t>Temperature-Induced Delay Drift in Xilinx FPGA Multi-gigabit Transceivers</t>
-  </si>
-  <si>
-    <t>Deep Learning–Based Real-Time Error Detection in Radiotherapy with EPID Images</t>
-  </si>
-  <si>
-    <t>High-dose-rate precise ionization chamber with real-time electronics for SC cyclotron-based proton therapy system</t>
-  </si>
-  <si>
-    <t>Realization of Large Model-Driven Tango Control and Data Interaction Analysis Tool</t>
-  </si>
-  <si>
-    <t>A Virtual Gamma-ray Spectrum Database for Training in Seawater Radioactivity Analysis</t>
-  </si>
-  <si>
-    <t>Optimising SiPM Array Architectures and Optical Coatings for High-Efficiency ZnSe(Al,O)–Based Strontium-90 Detection</t>
-  </si>
-  <si>
-    <t>Ion Irradiation facility with Performance Online Monitoring for High Temperature Superconducting Tape</t>
-  </si>
-  <si>
-    <t>The Realization of Ultra-High Dose Rate and Potential Frontier Applications on 230 MeV SC Cyclotron CYCIAE-230</t>
-  </si>
-  <si>
-    <t>AI Enhanced LLRF Controller for Ultra-lightweight SC Cyclotron CYCIAE-100B</t>
-  </si>
-  <si>
-    <t>Design of an Integrated Control System for Automated Operation of  Large Array of Imaging Atmospheric Cherenkov Telescope</t>
-  </si>
-  <si>
-    <t>Physics-Aware and Hardware-Efficient Federated Learning for Isotope Identification in Distributed Edge Radiation Networks</t>
-  </si>
-  <si>
-    <t>Design and Implementation of a Space Radiation Microdosimetric Detection Prototype</t>
-  </si>
-  <si>
-    <t>Design of Transmission Cable Delay Calibration Method for Large-Scale Electron Accelerators</t>
-  </si>
-  <si>
-    <t>Application of the FPGA Coprocessor TM FAST for Siemens S7-1500 PLCs in Neutron Instruments</t>
-  </si>
-  <si>
-    <t>A common framework for real-time structured data communication in fusion devices</t>
-  </si>
-  <si>
-    <t>Fueling modeling and control for ITER start of research operation</t>
-  </si>
-  <si>
-    <t>Jonathan Daniel</t>
-  </si>
-  <si>
-    <t>Emmanuel</t>
-  </si>
-  <si>
-    <t>Tianyi</t>
-  </si>
-  <si>
-    <t>Huang</t>
-  </si>
-  <si>
-    <t>Wanook</t>
-  </si>
-  <si>
-    <t>Arjana</t>
-  </si>
-  <si>
-    <t>Xiaofeng</t>
-  </si>
-  <si>
-    <t>Tianjue</t>
-  </si>
-  <si>
-    <t>Si</t>
-  </si>
-  <si>
-    <t>Yuxin</t>
-  </si>
-  <si>
-    <t>Xiaoyan</t>
-  </si>
-  <si>
-    <t>Haoqian</t>
-  </si>
-  <si>
-    <t>Harald</t>
-  </si>
-  <si>
-    <t>Nicolo</t>
-  </si>
-  <si>
-    <t>Eisch</t>
-  </si>
-  <si>
-    <t>Uwitonze</t>
-  </si>
-  <si>
-    <t>Jiang</t>
-  </si>
-  <si>
-    <t>Ji</t>
-  </si>
-  <si>
-    <t>Kolnikaj</t>
-  </si>
-  <si>
-    <t>Zhu</t>
-  </si>
-  <si>
-    <t>Ma</t>
-  </si>
-  <si>
-    <t>Gao</t>
-  </si>
-  <si>
-    <t>Kleines</t>
-  </si>
-  <si>
-    <t>Ferron</t>
-  </si>
-  <si>
-    <t>Weldon</t>
-  </si>
-  <si>
-    <t>Fermi National Accelerator Lab. (US)</t>
-  </si>
-  <si>
-    <t>National Institute for Nuclear Physics, Section of Pisa, Pisa, Italy</t>
-  </si>
-  <si>
-    <t>China Institute of Atomic Energy</t>
-  </si>
-  <si>
-    <t>IHEP - Chinese Academy of Sciences</t>
-  </si>
-  <si>
-    <t>Korea Atomic Energy Research Institute</t>
-  </si>
-  <si>
-    <t>University of Glasgow</t>
-  </si>
-  <si>
     <t>Tianjin University of Technology</t>
   </si>
   <si>
@@ -905,9 +860,6 @@
     <t>Universidad Politecnica de Madrid</t>
   </si>
   <si>
-    <t>INFN</t>
-  </si>
-  <si>
     <t>JLAB</t>
   </si>
   <si>
@@ -917,19 +869,16 @@
     <t>Hefei Institutes of Physical Science</t>
   </si>
   <si>
-    <t>University of California Irvine (US)</t>
-  </si>
-  <si>
-    <t>The University of Edinburgh (GB)</t>
-  </si>
-  <si>
-    <t>The Institute of High Energy Physics of the Chinese Academy of Sciences</t>
+    <t>University of California Irvine</t>
+  </si>
+  <si>
+    <t>The University of Edinburgh</t>
   </si>
   <si>
     <t>The University of Osaka</t>
   </si>
   <si>
-    <t>Universita e INFN, Padova (IT)</t>
+    <t>Universita e INFN Padova</t>
   </si>
   <si>
     <t>Shape-factor analysis of real-time, in-situ photon-depth spectra for land quality β--emitter assay</t>
@@ -971,9 +920,6 @@
     <t>UPGRADED CONTROL SYSTEM FOR THE ELECTRON CYCLOTRON HEATING EXPANSION SYSTEM ON EAST</t>
   </si>
   <si>
-    <t>Development of a Portable Real-Time Radiation Measurement Technology for Digital Twin Based Plant Situation Monitoring</t>
-  </si>
-  <si>
     <t>Data Orchestration and Large Model-Driven Interactive Diagnosis for LHAASO Operational Data</t>
   </si>
   <si>
@@ -1013,9 +959,6 @@
     <t>Weiye</t>
   </si>
   <si>
-    <t>Hyeoung Woo</t>
-  </si>
-  <si>
     <t>Heru</t>
   </si>
   <si>
@@ -1043,19 +986,13 @@
     <t>Gioiosa</t>
   </si>
   <si>
-    <t>Park</t>
-  </si>
-  <si>
     <t>Guo</t>
   </si>
   <si>
     <t>Lancaster University</t>
   </si>
   <si>
-    <t>Justus-Liebig-Universitaet Giessen (DE)</t>
-  </si>
-  <si>
-    <t>IHEP</t>
+    <t>Justus-Liebig-Universitaet Giessen</t>
   </si>
   <si>
     <t>INFN Napoli</t>
@@ -1079,9 +1016,6 @@
     <t>Institute of Energy Hefei Comprehensive National Science Center</t>
   </si>
   <si>
-    <t>Central Research Institute, Korea Hydro &amp; Nuclear Power Co., Ltd.</t>
-  </si>
-  <si>
     <t>Institute of Energy, Hefei Comprehensive National Science Center</t>
   </si>
   <si>
@@ -1109,12 +1043,6 @@
     <t>A Full on-Chip LDO Regulator with self-adapting compensation networks for Front-end Readout Circuit</t>
   </si>
   <si>
-    <t>The μMUX readout electronic system of the AliCPT</t>
-  </si>
-  <si>
-    <t>Low-Noise Room-Temperature Readout Electronics for TDM-SQUID TES Arrays in the AliCPT-40G Telescope</t>
-  </si>
-  <si>
     <t>A 14-bit 100 Ms/s Pipeline ADC for Silicon Pixel Sensor in Gaseous Detectors</t>
   </si>
   <si>
@@ -1145,12 +1073,6 @@
     <t>Xiayu</t>
   </si>
   <si>
-    <t>Xiangxiang</t>
-  </si>
-  <si>
-    <t>Tangchong</t>
-  </si>
-  <si>
     <t>Haoqing</t>
   </si>
   <si>
@@ -1169,12 +1091,6 @@
     <t>Sun</t>
   </si>
   <si>
-    <t>Ren</t>
-  </si>
-  <si>
-    <t>Kuang</t>
-  </si>
-  <si>
     <t>Xie</t>
   </si>
   <si>
@@ -1184,15 +1100,12 @@
     <t>ITE</t>
   </si>
   <si>
-    <t>Instituto de Física Corpuscular (CSIC-UV)</t>
+    <t>Instituto de Física Corpuscular</t>
   </si>
   <si>
     <t>Northwestern Polytechnical University</t>
   </si>
   <si>
-    <t>SHANDONG University</t>
-  </si>
-  <si>
     <t>Institute of Modern Physics, Chinese Academy of Sciences</t>
   </si>
   <si>
@@ -1337,43 +1250,28 @@
     <t>Kobayashi</t>
   </si>
   <si>
-    <t>Università di Padova/Consorzio RFX</t>
-  </si>
-  <si>
     <t>Forschungszentrum Jülich GmbH, ITE</t>
   </si>
   <si>
-    <t>IHEP, UCAS</t>
-  </si>
-  <si>
-    <t>Institute of Plasma Physics,Chinese Academy of Sciences</t>
-  </si>
-  <si>
-    <t>中国科学院高能物理研究所</t>
-  </si>
-  <si>
-    <t>University of Zurich (CH)</t>
+    <t>University of Zurich</t>
   </si>
   <si>
     <t>Università di Pisa</t>
   </si>
   <si>
-    <t>University of Sussex (GB)</t>
+    <t>University of Sussex</t>
   </si>
   <si>
     <t>University of Pisa</t>
   </si>
   <si>
-    <t>Institute of High Energy Physics (IHEP), Chinese Academy of Sciences</t>
-  </si>
-  <si>
-    <t>University of Notre Dame (US)</t>
+    <t>University of Notre Dame</t>
   </si>
   <si>
     <t>Department of Physics, University of Pisa</t>
   </si>
   <si>
-    <t>ETH Zurich (CH)</t>
+    <t>ETH Zurich</t>
   </si>
   <si>
     <t>Research Center for Nuclear Physics</t>
@@ -1467,6 +1365,12 @@
   </si>
   <si>
     <t>pi5pm28</t>
+  </si>
+  <si>
+    <t>Universite Libre de Bruxelles</t>
+  </si>
+  <si>
+    <t>INFN Genova</t>
   </si>
 </sst>
 </file>
@@ -1836,7 +1740,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>449</v>
+        <v>415</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1844,7 +1748,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>450</v>
+        <v>416</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1907,16 +1811,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>351</v>
+        <v>329</v>
       </c>
       <c r="D2" t="s">
-        <v>364</v>
+        <v>340</v>
       </c>
       <c r="E2" t="s">
-        <v>375</v>
+        <v>349</v>
       </c>
       <c r="F2" t="s">
-        <v>383</v>
+        <v>355</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1927,16 +1831,16 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
       <c r="D3" t="s">
-        <v>365</v>
+        <v>341</v>
       </c>
       <c r="E3" t="s">
-        <v>376</v>
+        <v>350</v>
       </c>
       <c r="F3" t="s">
-        <v>384</v>
+        <v>356</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1947,16 +1851,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>353</v>
+        <v>331</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F4" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -1967,16 +1871,16 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>354</v>
+        <v>332</v>
       </c>
       <c r="D5" t="s">
-        <v>366</v>
+        <v>342</v>
       </c>
       <c r="E5" t="s">
-        <v>377</v>
+        <v>351</v>
       </c>
       <c r="F5" t="s">
-        <v>254</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1987,16 +1891,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>355</v>
+        <v>333</v>
       </c>
       <c r="D6" t="s">
-        <v>367</v>
+        <v>343</v>
       </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F6" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -2007,16 +1911,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>356</v>
+        <v>334</v>
       </c>
       <c r="D7" t="s">
-        <v>368</v>
+        <v>344</v>
       </c>
       <c r="E7" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="F7" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -2027,16 +1931,16 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>357</v>
+        <v>335</v>
       </c>
       <c r="D8" t="s">
-        <v>369</v>
+        <v>345</v>
       </c>
       <c r="E8" t="s">
-        <v>378</v>
+        <v>352</v>
       </c>
       <c r="F8" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -2047,117 +1951,83 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>358</v>
+        <v>336</v>
       </c>
       <c r="D9" t="s">
-        <v>370</v>
+        <v>346</v>
       </c>
       <c r="E9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F9" t="s">
-        <v>385</v>
+        <v>357</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>359</v>
+        <v>337</v>
       </c>
       <c r="D10" t="s">
-        <v>371</v>
+        <v>347</v>
       </c>
       <c r="E10" t="s">
-        <v>379</v>
+        <v>353</v>
       </c>
       <c r="F10" t="s">
-        <v>136</v>
+        <v>358</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="B11" s="1">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>360</v>
+        <v>338</v>
       </c>
       <c r="D11" t="s">
-        <v>372</v>
+        <v>348</v>
       </c>
       <c r="E11" t="s">
-        <v>380</v>
+        <v>354</v>
       </c>
       <c r="F11" t="s">
-        <v>386</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="B12" s="1">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>361</v>
+        <v>339</v>
       </c>
       <c r="D12" t="s">
-        <v>373</v>
+        <v>347</v>
       </c>
       <c r="E12" t="s">
-        <v>381</v>
+        <v>353</v>
       </c>
       <c r="F12" t="s">
-        <v>387</v>
+        <v>358</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>194</v>
-      </c>
-      <c r="B13" s="1">
-        <v>12</v>
-      </c>
-      <c r="C13" t="s">
-        <v>362</v>
-      </c>
-      <c r="D13" t="s">
-        <v>374</v>
-      </c>
-      <c r="E13" t="s">
-        <v>382</v>
-      </c>
-      <c r="F13" t="s">
-        <v>151</v>
-      </c>
+      <c r="B13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>200</v>
-      </c>
-      <c r="B14" s="1">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s">
-        <v>363</v>
-      </c>
-      <c r="D14" t="s">
-        <v>373</v>
-      </c>
-      <c r="E14" t="s">
-        <v>381</v>
-      </c>
-      <c r="F14" t="s">
-        <v>387</v>
-      </c>
+      <c r="B14" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2200,356 +2070,356 @@
         <v>73</v>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>388</v>
+        <v>359</v>
       </c>
       <c r="D2" t="s">
-        <v>406</v>
+        <v>377</v>
       </c>
       <c r="E2" t="s">
-        <v>422</v>
+        <v>393</v>
       </c>
       <c r="F2" t="s">
-        <v>435</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>115</v>
       </c>
-      <c r="B3">
-        <v>14</v>
+      <c r="B3" s="1">
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>389</v>
+        <v>360</v>
       </c>
       <c r="D3" t="s">
-        <v>407</v>
+        <v>378</v>
       </c>
       <c r="E3" t="s">
-        <v>423</v>
+        <v>394</v>
       </c>
       <c r="F3" t="s">
-        <v>436</v>
+        <v>406</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>134</v>
       </c>
-      <c r="B4">
-        <v>15</v>
+      <c r="B4" s="1">
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>390</v>
+        <v>361</v>
       </c>
       <c r="D4" t="s">
-        <v>408</v>
+        <v>379</v>
       </c>
       <c r="E4" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F4" t="s">
-        <v>437</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>136</v>
       </c>
-      <c r="B5">
-        <v>16</v>
+      <c r="B5" s="1">
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>391</v>
+        <v>362</v>
       </c>
       <c r="D5" t="s">
-        <v>409</v>
+        <v>380</v>
       </c>
       <c r="E5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F5" t="s">
-        <v>438</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>139</v>
       </c>
-      <c r="B6">
-        <v>17</v>
+      <c r="B6" s="1">
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>392</v>
+        <v>363</v>
       </c>
       <c r="D6" t="s">
-        <v>410</v>
+        <v>381</v>
       </c>
       <c r="E6" t="s">
-        <v>424</v>
+        <v>395</v>
       </c>
       <c r="F6" t="s">
-        <v>439</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>147</v>
       </c>
-      <c r="B7">
-        <v>18</v>
+      <c r="B7" s="1">
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>393</v>
+        <v>364</v>
       </c>
       <c r="D7" t="s">
-        <v>411</v>
+        <v>382</v>
       </c>
       <c r="E7" t="s">
-        <v>425</v>
+        <v>396</v>
       </c>
       <c r="F7" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>148</v>
       </c>
-      <c r="B8">
-        <v>19</v>
+      <c r="B8" s="1">
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>394</v>
+        <v>365</v>
       </c>
       <c r="D8" t="s">
-        <v>412</v>
+        <v>383</v>
       </c>
       <c r="E8" t="s">
-        <v>426</v>
+        <v>397</v>
       </c>
       <c r="F8" t="s">
-        <v>440</v>
+        <v>407</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>149</v>
       </c>
-      <c r="B9">
-        <v>20</v>
+      <c r="B9" s="1">
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>395</v>
+        <v>366</v>
       </c>
       <c r="D9" t="s">
-        <v>413</v>
+        <v>384</v>
       </c>
       <c r="E9" t="s">
-        <v>427</v>
+        <v>398</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>150</v>
       </c>
-      <c r="B10">
-        <v>21</v>
+      <c r="B10" s="1">
+        <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>396</v>
+        <v>367</v>
       </c>
       <c r="D10" t="s">
-        <v>414</v>
+        <v>385</v>
       </c>
       <c r="E10" t="s">
-        <v>428</v>
+        <v>399</v>
       </c>
       <c r="F10" t="s">
-        <v>441</v>
+        <v>408</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>153</v>
       </c>
-      <c r="B11">
-        <v>22</v>
+      <c r="B11" s="1">
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>397</v>
+        <v>368</v>
       </c>
       <c r="D11" t="s">
-        <v>321</v>
+        <v>303</v>
       </c>
       <c r="E11" t="s">
-        <v>429</v>
+        <v>400</v>
       </c>
       <c r="F11" t="s">
-        <v>442</v>
+        <v>409</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>173</v>
       </c>
-      <c r="B12">
-        <v>23</v>
+      <c r="B12" s="1">
+        <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>398</v>
+        <v>369</v>
       </c>
       <c r="D12" t="s">
-        <v>415</v>
+        <v>386</v>
       </c>
       <c r="E12" t="s">
-        <v>430</v>
+        <v>401</v>
       </c>
       <c r="F12" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>189</v>
       </c>
-      <c r="B13">
-        <v>24</v>
+      <c r="B13" s="1">
+        <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>399</v>
+        <v>370</v>
       </c>
       <c r="D13" t="s">
-        <v>416</v>
+        <v>387</v>
       </c>
       <c r="E13" t="s">
-        <v>431</v>
+        <v>402</v>
       </c>
       <c r="F13" t="s">
-        <v>443</v>
+        <v>410</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>192</v>
       </c>
-      <c r="B14">
-        <v>25</v>
+      <c r="B14" s="1">
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>400</v>
+        <v>371</v>
       </c>
       <c r="D14" t="s">
-        <v>417</v>
+        <v>388</v>
       </c>
       <c r="E14" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F14" t="s">
-        <v>444</v>
+        <v>142</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>197</v>
       </c>
-      <c r="B15">
-        <v>26</v>
+      <c r="B15" s="1">
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>401</v>
+        <v>372</v>
       </c>
       <c r="D15" t="s">
-        <v>418</v>
+        <v>389</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F15" t="s">
-        <v>445</v>
+        <v>411</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>199</v>
       </c>
-      <c r="B16">
-        <v>27</v>
+      <c r="B16" s="1">
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>402</v>
+        <v>373</v>
       </c>
       <c r="D16" t="s">
-        <v>419</v>
+        <v>390</v>
       </c>
       <c r="E16" t="s">
-        <v>432</v>
+        <v>403</v>
       </c>
       <c r="F16" t="s">
-        <v>446</v>
+        <v>412</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>207</v>
       </c>
-      <c r="B17">
-        <v>28</v>
+      <c r="B17" s="1">
+        <v>27</v>
       </c>
       <c r="C17" t="s">
-        <v>403</v>
+        <v>374</v>
       </c>
       <c r="D17" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E17" t="s">
-        <v>381</v>
+        <v>353</v>
       </c>
       <c r="F17" t="s">
-        <v>447</v>
+        <v>413</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>213</v>
       </c>
-      <c r="B18">
-        <v>13</v>
+      <c r="B18" s="1">
+        <v>28</v>
       </c>
       <c r="C18" t="s">
+        <v>375</v>
+      </c>
+      <c r="D18" t="s">
+        <v>391</v>
+      </c>
+      <c r="E18" t="s">
         <v>404</v>
       </c>
-      <c r="D18" t="s">
-        <v>420</v>
-      </c>
-      <c r="E18" t="s">
-        <v>433</v>
-      </c>
       <c r="F18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>216</v>
       </c>
-      <c r="B19">
-        <v>17</v>
+      <c r="B19" s="1">
+        <v>13</v>
       </c>
       <c r="C19" t="s">
+        <v>376</v>
+      </c>
+      <c r="D19" t="s">
+        <v>392</v>
+      </c>
+      <c r="E19" t="s">
         <v>405</v>
       </c>
-      <c r="D19" t="s">
-        <v>421</v>
-      </c>
-      <c r="E19" t="s">
-        <v>434</v>
-      </c>
       <c r="F19" t="s">
-        <v>448</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>
@@ -2716,7 +2586,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>451</v>
+        <v>417</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2724,7 +2594,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>452</v>
+        <v>418</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -2732,7 +2602,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>453</v>
+        <v>419</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -2740,7 +2610,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>454</v>
+        <v>420</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -2748,7 +2618,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>455</v>
+        <v>421</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -2756,7 +2626,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>456</v>
+        <v>422</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -2764,7 +2634,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>457</v>
+        <v>423</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -2772,7 +2642,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>458</v>
+        <v>424</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -2780,7 +2650,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>459</v>
+        <v>425</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -2788,7 +2658,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>460</v>
+        <v>426</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -2796,7 +2666,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>461</v>
+        <v>427</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -2804,7 +2674,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>462</v>
+        <v>428</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -2812,7 +2682,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>463</v>
+        <v>429</v>
       </c>
       <c r="B14">
         <v>13</v>
@@ -2820,7 +2690,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>464</v>
+        <v>430</v>
       </c>
       <c r="B15">
         <v>14</v>
@@ -2828,7 +2698,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>465</v>
+        <v>431</v>
       </c>
       <c r="B16">
         <v>15</v>
@@ -2836,7 +2706,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>466</v>
+        <v>432</v>
       </c>
       <c r="B17">
         <v>16</v>
@@ -2844,7 +2714,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>467</v>
+        <v>433</v>
       </c>
       <c r="B18">
         <v>17</v>
@@ -2852,7 +2722,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>468</v>
+        <v>434</v>
       </c>
       <c r="B19">
         <v>18</v>
@@ -2860,7 +2730,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>469</v>
+        <v>435</v>
       </c>
       <c r="B20">
         <v>19</v>
@@ -2868,7 +2738,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>470</v>
+        <v>436</v>
       </c>
       <c r="B21">
         <v>20</v>
@@ -2876,7 +2746,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>471</v>
+        <v>437</v>
       </c>
       <c r="B22">
         <v>21</v>
@@ -2884,7 +2754,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>472</v>
+        <v>438</v>
       </c>
       <c r="B23">
         <v>22</v>
@@ -2892,7 +2762,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>473</v>
+        <v>439</v>
       </c>
       <c r="B24">
         <v>23</v>
@@ -2900,7 +2770,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>474</v>
+        <v>440</v>
       </c>
       <c r="B25">
         <v>24</v>
@@ -2908,7 +2778,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>475</v>
+        <v>441</v>
       </c>
       <c r="B26">
         <v>25</v>
@@ -2916,7 +2786,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>476</v>
+        <v>442</v>
       </c>
       <c r="B27">
         <v>26</v>
@@ -2924,7 +2794,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>477</v>
+        <v>443</v>
       </c>
       <c r="B28">
         <v>27</v>
@@ -2932,7 +2802,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>478</v>
+        <v>444</v>
       </c>
       <c r="B29">
         <v>28</v>
@@ -2945,7 +2815,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12.6640625" customWidth="1"/>
@@ -2985,13 +2855,13 @@
         <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -3005,13 +2875,13 @@
         <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -3025,13 +2895,13 @@
         <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -3045,13 +2915,13 @@
         <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -3065,33 +2935,13 @@
         <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>204</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -3138,16 +2988,16 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F2" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -3158,16 +3008,16 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F3" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -3178,16 +3028,16 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F4" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -3198,16 +3048,16 @@
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F5" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -3218,16 +3068,16 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F6" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -3238,16 +3088,16 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E7" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F7" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -3258,16 +3108,16 @@
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F8" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -3278,16 +3128,16 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F9" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -3298,16 +3148,16 @@
         <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D10" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F10" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -3318,16 +3168,16 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E11" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F11" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -3338,16 +3188,16 @@
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D12" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E12" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F12" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -3358,16 +3208,16 @@
         <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F13" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -3378,16 +3228,16 @@
         <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D14" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E14" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F14" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -3398,16 +3248,16 @@
         <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D15" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E15" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F15" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -3418,16 +3268,16 @@
         <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D16" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="F16" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -3438,16 +3288,16 @@
         <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D17" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E17" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F17" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -3458,16 +3308,16 @@
         <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E18" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F18" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -3478,13 +3328,16 @@
         <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D19" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E19" t="s">
-        <v>128</v>
+        <v>123</v>
+      </c>
+      <c r="F19" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -3495,13 +3348,13 @@
         <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D20" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E20" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -3512,16 +3365,16 @@
         <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D21" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E21" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F21" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -3532,16 +3385,16 @@
         <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D22" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E22" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F22" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -3552,16 +3405,16 @@
         <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D23" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E23" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="F23" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -3572,16 +3425,16 @@
         <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E24" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F24" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -3592,16 +3445,16 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D25" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E25" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F25" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -3612,16 +3465,16 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D26" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E26" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F26" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -3632,16 +3485,16 @@
         <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D27" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E27" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F27" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -3652,16 +3505,16 @@
         <v>18</v>
       </c>
       <c r="C28" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D28" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E28" t="s">
+        <v>129</v>
+      </c>
+      <c r="F28" t="s">
         <v>134</v>
-      </c>
-      <c r="F28" t="s">
-        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -3671,7 +3524,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12.6640625" customWidth="1"/>
@@ -3708,16 +3561,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="D2" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="E2" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="F2" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -3728,287 +3581,250 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="D3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E3" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="F3" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="D4" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="E4" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="F4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="D5" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="E5" t="s">
-        <v>187</v>
+        <v>129</v>
       </c>
       <c r="F5" t="s">
-        <v>151</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="D6" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="F6" t="s">
-        <v>198</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D7" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E7" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="F7" t="s">
-        <v>143</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D8" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="E8" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="F8" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="D9" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="E9" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="F9" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="B10">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D10" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="E10" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="F10" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="B11">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="D11" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="E11" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="F11" t="s">
-        <v>202</v>
+        <v>445</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="B12">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D12" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E12" t="s">
-        <v>192</v>
+        <v>125</v>
       </c>
       <c r="F12" t="s">
-        <v>203</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>161</v>
+        <v>196</v>
       </c>
       <c r="B13">
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="D13" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="E13" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="F13" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>165</v>
+        <v>218</v>
       </c>
       <c r="B14">
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D14" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="E14" t="s">
-        <v>130</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>196</v>
+        <v>219</v>
       </c>
       <c r="B15">
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D15" t="s">
+        <v>172</v>
+      </c>
+      <c r="E15" t="s">
         <v>182</v>
-      </c>
-      <c r="E15" t="s">
-        <v>194</v>
-      </c>
-      <c r="F15" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>218</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16" t="s">
-        <v>167</v>
-      </c>
-      <c r="D16" t="s">
-        <v>183</v>
-      </c>
-      <c r="E16" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>219</v>
-      </c>
-      <c r="B17">
-        <v>5</v>
-      </c>
-      <c r="C17" t="s">
-        <v>168</v>
-      </c>
-      <c r="D17" t="s">
-        <v>183</v>
-      </c>
-      <c r="E17" t="s">
-        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -4055,16 +3871,16 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="D2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E2" t="s">
         <v>223</v>
       </c>
-      <c r="E2" t="s">
-        <v>237</v>
-      </c>
       <c r="F2" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4075,16 +3891,16 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="D3" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="E3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -4095,16 +3911,16 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="D4" t="s">
+        <v>210</v>
+      </c>
+      <c r="E4" t="s">
         <v>224</v>
       </c>
-      <c r="E4" t="s">
-        <v>238</v>
-      </c>
       <c r="F4" t="s">
-        <v>249</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4115,16 +3931,16 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="D5" t="s">
+        <v>211</v>
+      </c>
+      <c r="E5" t="s">
         <v>225</v>
       </c>
-      <c r="E5" t="s">
-        <v>239</v>
-      </c>
       <c r="F5" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -4135,16 +3951,16 @@
         <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="D6" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F6" t="s">
-        <v>251</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -4155,16 +3971,16 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="D7" t="s">
-        <v>227</v>
+        <v>213</v>
       </c>
       <c r="E7" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="F7" t="s">
-        <v>252</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -4175,16 +3991,16 @@
         <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="D8" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
       <c r="E8" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="F8" t="s">
-        <v>253</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -4195,16 +4011,16 @@
         <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="D9" t="s">
-        <v>229</v>
+        <v>215</v>
       </c>
       <c r="E9" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="F9" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -4215,16 +4031,16 @@
         <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="D10" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="E10" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F10" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -4235,16 +4051,16 @@
         <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="D11" t="s">
+        <v>211</v>
+      </c>
+      <c r="E11" t="s">
         <v>225</v>
       </c>
-      <c r="E11" t="s">
-        <v>239</v>
-      </c>
       <c r="F11" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -4255,16 +4071,16 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="D12" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="E12" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="F12" t="s">
-        <v>149</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -4275,16 +4091,16 @@
         <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="D13" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="E13" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F13" t="s">
-        <v>254</v>
+        <v>239</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -4295,16 +4111,16 @@
         <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="D14" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="E14" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="F14" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -4315,16 +4131,16 @@
         <v>28</v>
       </c>
       <c r="C15" t="s">
-        <v>219</v>
+        <v>205</v>
       </c>
       <c r="D15" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="E15" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F15" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -4335,16 +4151,16 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="D16" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="E16" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="F16" t="s">
-        <v>255</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -4355,16 +4171,16 @@
         <v>19</v>
       </c>
       <c r="C17" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="D17" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="E17" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="F17" t="s">
-        <v>256</v>
+        <v>241</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -4375,16 +4191,16 @@
         <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="D18" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E18" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
       <c r="F18" t="s">
-        <v>257</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -4431,16 +4247,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>258</v>
+        <v>243</v>
       </c>
       <c r="D2" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="E2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4451,16 +4267,16 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="D3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E3" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="F3" t="s">
-        <v>290</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -4471,16 +4287,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="D4" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="E4" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="F4" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4491,16 +4307,16 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>261</v>
+        <v>246</v>
       </c>
       <c r="D5" t="s">
-        <v>273</v>
+        <v>258</v>
       </c>
       <c r="E5" t="s">
-        <v>283</v>
+        <v>268</v>
       </c>
       <c r="F5" t="s">
-        <v>291</v>
+        <v>446</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -4511,16 +4327,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E6" t="s">
-        <v>284</v>
+        <v>269</v>
       </c>
       <c r="F6" t="s">
-        <v>292</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -4531,16 +4347,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="D7" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="E7" t="s">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="F7" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -4551,16 +4367,16 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="D8" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="E8" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F8" t="s">
-        <v>294</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -4571,16 +4387,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>265</v>
+        <v>250</v>
       </c>
       <c r="D9" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="E9" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="F9" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -4591,16 +4407,16 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>266</v>
+        <v>251</v>
       </c>
       <c r="D10" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="E10" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="F10" t="s">
-        <v>296</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -4611,16 +4427,16 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>267</v>
+        <v>252</v>
       </c>
       <c r="D11" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E11" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F11" t="s">
-        <v>297</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -4631,16 +4447,16 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="D12" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="E12" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="F12" t="s">
-        <v>298</v>
+        <v>281</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -4651,16 +4467,16 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>269</v>
+        <v>254</v>
       </c>
       <c r="D13" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="E13" t="s">
-        <v>289</v>
+        <v>274</v>
       </c>
       <c r="F13" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -4671,16 +4487,16 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>270</v>
+        <v>255</v>
       </c>
       <c r="D14" t="s">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="E14" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F14" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -4690,7 +4506,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12.6640625" customWidth="1"/>
@@ -4727,16 +4543,16 @@
         <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
       <c r="D2" t="s">
-        <v>316</v>
+        <v>298</v>
       </c>
       <c r="E2" t="s">
-        <v>329</v>
+        <v>310</v>
       </c>
       <c r="F2" t="s">
-        <v>339</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4747,16 +4563,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>301</v>
+        <v>284</v>
       </c>
       <c r="D3" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="E3" t="s">
-        <v>330</v>
+        <v>311</v>
       </c>
       <c r="F3" t="s">
-        <v>340</v>
+        <v>320</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -4767,16 +4583,16 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>302</v>
+        <v>285</v>
       </c>
       <c r="D4" t="s">
-        <v>318</v>
+        <v>300</v>
       </c>
       <c r="E4" t="s">
-        <v>331</v>
+        <v>312</v>
       </c>
       <c r="F4" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4787,16 +4603,16 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>303</v>
+        <v>286</v>
       </c>
       <c r="D5" t="s">
-        <v>319</v>
+        <v>301</v>
       </c>
       <c r="E5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F5" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -4807,16 +4623,16 @@
         <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>304</v>
+        <v>287</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E6" t="s">
-        <v>332</v>
+        <v>313</v>
       </c>
       <c r="F6" t="s">
-        <v>342</v>
+        <v>321</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -4827,16 +4643,16 @@
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="D7" t="s">
-        <v>320</v>
+        <v>302</v>
       </c>
       <c r="E7" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="F7" t="s">
-        <v>343</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -4847,16 +4663,16 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>306</v>
+        <v>289</v>
       </c>
       <c r="D8" t="s">
-        <v>321</v>
+        <v>303</v>
       </c>
       <c r="E8" t="s">
-        <v>333</v>
+        <v>314</v>
       </c>
       <c r="F8" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -4867,16 +4683,16 @@
         <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>307</v>
+        <v>290</v>
       </c>
       <c r="D9" t="s">
-        <v>322</v>
+        <v>304</v>
       </c>
       <c r="E9" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
       <c r="F9" t="s">
-        <v>344</v>
+        <v>323</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -4887,16 +4703,16 @@
         <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>308</v>
+        <v>291</v>
       </c>
       <c r="D10" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
       <c r="E10" t="s">
-        <v>335</v>
+        <v>316</v>
       </c>
       <c r="F10" t="s">
-        <v>345</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -4907,16 +4723,16 @@
         <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>309</v>
+        <v>292</v>
       </c>
       <c r="D11" t="s">
-        <v>324</v>
+        <v>306</v>
       </c>
       <c r="E11" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="F11" t="s">
-        <v>346</v>
+        <v>325</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -4927,16 +4743,16 @@
         <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>310</v>
+        <v>293</v>
       </c>
       <c r="D12" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="E12" t="s">
-        <v>336</v>
+        <v>317</v>
       </c>
       <c r="F12" t="s">
-        <v>347</v>
+        <v>326</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -4947,16 +4763,16 @@
         <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>311</v>
+        <v>294</v>
       </c>
       <c r="D13" t="s">
-        <v>325</v>
+        <v>307</v>
       </c>
       <c r="E13" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F13" t="s">
-        <v>348</v>
+        <v>327</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -4967,76 +4783,56 @@
         <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>312</v>
+        <v>295</v>
       </c>
       <c r="D14" t="s">
-        <v>326</v>
+        <v>308</v>
       </c>
       <c r="E14" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F14" t="s">
-        <v>343</v>
+        <v>322</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="B15">
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>313</v>
+        <v>296</v>
       </c>
       <c r="D15" t="s">
-        <v>327</v>
+        <v>212</v>
       </c>
       <c r="E15" t="s">
-        <v>337</v>
+        <v>129</v>
       </c>
       <c r="F15" t="s">
-        <v>349</v>
+        <v>142</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B16">
         <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>314</v>
+        <v>297</v>
       </c>
       <c r="D16" t="s">
-        <v>226</v>
+        <v>309</v>
       </c>
       <c r="E16" t="s">
-        <v>134</v>
+        <v>318</v>
       </c>
       <c r="F16" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>128</v>
-      </c>
-      <c r="B17">
-        <v>14</v>
-      </c>
-      <c r="C17" t="s">
-        <v>315</v>
-      </c>
-      <c r="D17" t="s">
         <v>328</v>
-      </c>
-      <c r="E17" t="s">
-        <v>338</v>
-      </c>
-      <c r="F17" t="s">
-        <v>350</v>
       </c>
     </row>
   </sheetData>

</xml_diff>